<commit_message>
feat: leverage-aware diversification — max_stack_exposure 0.35, implied total floor 4.5, proper leverage scoring, ownership display fix
</commit_message>
<xml_diff>
--- a/data/live/BallparkPal_Batters_2026-04-12.xlsx
+++ b/data/live/BallparkPal_Batters_2026-04-12.xlsx
@@ -23947,61 +23947,61 @@
         <v>5</v>
       </c>
       <c r="L218" t="n">
-        <v>4.419</v>
+        <v>4.405</v>
       </c>
       <c r="M218" t="n">
-        <v>3.852</v>
+        <v>3.823</v>
       </c>
       <c r="N218" t="n">
-        <v>0.964</v>
+        <v>0.944</v>
       </c>
       <c r="O218" t="n">
-        <v>1.815</v>
+        <v>1.737</v>
       </c>
       <c r="P218" t="n">
-        <v>1.021</v>
+        <v>1.015</v>
       </c>
       <c r="Q218" t="n">
-        <v>0.479</v>
+        <v>0.495</v>
       </c>
       <c r="R218" t="n">
-        <v>0.508</v>
+        <v>0.504</v>
       </c>
       <c r="S218" t="n">
-        <v>0.255</v>
+        <v>0.259</v>
       </c>
       <c r="T218" t="n">
-        <v>0.007</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="U218" t="n">
-        <v>0.194</v>
+        <v>0.172</v>
       </c>
       <c r="V218" t="n">
-        <v>0.617</v>
+        <v>0.591</v>
       </c>
       <c r="W218" t="n">
-        <v>0.639</v>
+        <v>0.599</v>
       </c>
       <c r="X218" t="n">
-        <v>0.031</v>
+        <v>0.041</v>
       </c>
       <c r="Y218" t="n">
-        <v>0.026</v>
+        <v>0.036</v>
       </c>
       <c r="Z218" t="n">
-        <v>8.391</v>
+        <v>8.146000000000001</v>
       </c>
       <c r="AA218" t="n">
-        <v>11.237</v>
+        <v>10.893</v>
       </c>
       <c r="AB218" t="n">
-        <v>0.178</v>
+        <v>0.16</v>
       </c>
       <c r="AC218" t="n">
-        <v>0.651</v>
+        <v>0.654</v>
       </c>
       <c r="AD218" t="n">
-        <v>0.026</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="219">
@@ -24055,61 +24055,61 @@
         <v>3</v>
       </c>
       <c r="L219" t="n">
-        <v>4.589</v>
+        <v>4.575</v>
       </c>
       <c r="M219" t="n">
-        <v>3.727</v>
+        <v>3.731</v>
       </c>
       <c r="N219" t="n">
-        <v>0.995</v>
+        <v>1.011</v>
       </c>
       <c r="O219" t="n">
-        <v>1.648</v>
+        <v>1.599</v>
       </c>
       <c r="P219" t="n">
-        <v>0.702</v>
+        <v>0.696</v>
       </c>
       <c r="Q219" t="n">
-        <v>0.755</v>
+        <v>0.741</v>
       </c>
       <c r="R219" t="n">
-        <v>0.643</v>
+        <v>0.681</v>
       </c>
       <c r="S219" t="n">
-        <v>0.196</v>
+        <v>0.195</v>
       </c>
       <c r="T219" t="n">
-        <v>0.008</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="U219" t="n">
-        <v>0.147</v>
+        <v>0.125</v>
       </c>
       <c r="V219" t="n">
-        <v>0.608</v>
+        <v>0.548</v>
       </c>
       <c r="W219" t="n">
-        <v>0.707</v>
+        <v>0.649</v>
       </c>
       <c r="X219" t="n">
         <v>0.048</v>
       </c>
       <c r="Y219" t="n">
-        <v>0.04</v>
+        <v>0.038</v>
       </c>
       <c r="Z219" t="n">
-        <v>8.785</v>
+        <v>8.41</v>
       </c>
       <c r="AA219" t="n">
-        <v>11.838</v>
+        <v>11.244</v>
       </c>
       <c r="AB219" t="n">
-        <v>0.137</v>
+        <v>0.116</v>
       </c>
       <c r="AC219" t="n">
-        <v>0.654</v>
+        <v>0.672</v>
       </c>
       <c r="AD219" t="n">
-        <v>0.039</v>
+        <v>0.037</v>
       </c>
     </row>
     <row r="220">
@@ -24160,64 +24160,64 @@
         </is>
       </c>
       <c r="K220" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L220" t="n">
-        <v>4.23</v>
+        <v>4.324</v>
       </c>
       <c r="M220" t="n">
-        <v>3.583</v>
+        <v>3.649</v>
       </c>
       <c r="N220" t="n">
-        <v>0.923</v>
+        <v>0.914</v>
       </c>
       <c r="O220" t="n">
-        <v>1.738</v>
+        <v>1.692</v>
       </c>
       <c r="P220" t="n">
-        <v>1.049</v>
+        <v>1.104</v>
       </c>
       <c r="Q220" t="n">
-        <v>0.554</v>
+        <v>0.599</v>
       </c>
       <c r="R220" t="n">
-        <v>0.507</v>
+        <v>0.51</v>
       </c>
       <c r="S220" t="n">
-        <v>0.213</v>
+        <v>0.214</v>
       </c>
       <c r="T220" t="n">
         <v>0.006</v>
       </c>
       <c r="U220" t="n">
-        <v>0.197</v>
+        <v>0.184</v>
       </c>
       <c r="V220" t="n">
-        <v>0.651</v>
+        <v>0.681</v>
       </c>
       <c r="W220" t="n">
-        <v>0.633</v>
+        <v>0.608</v>
       </c>
       <c r="X220" t="n">
-        <v>0.016</v>
+        <v>0.023</v>
       </c>
       <c r="Y220" t="n">
-        <v>0.013</v>
+        <v>0.018</v>
       </c>
       <c r="Z220" t="n">
-        <v>8.34</v>
+        <v>8.353</v>
       </c>
       <c r="AA220" t="n">
-        <v>11.255</v>
+        <v>11.308</v>
       </c>
       <c r="AB220" t="n">
-        <v>0.18</v>
+        <v>0.165</v>
       </c>
       <c r="AC220" t="n">
-        <v>0.631</v>
+        <v>0.626</v>
       </c>
       <c r="AD220" t="n">
-        <v>0.012</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="221">
@@ -24268,64 +24268,64 @@
         </is>
       </c>
       <c r="K221" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L221" t="n">
-        <v>4.017</v>
+        <v>4.151</v>
       </c>
       <c r="M221" t="n">
-        <v>3.361</v>
+        <v>3.485</v>
       </c>
       <c r="N221" t="n">
-        <v>0.803</v>
+        <v>0.836</v>
       </c>
       <c r="O221" t="n">
-        <v>1.518</v>
+        <v>1.558</v>
       </c>
       <c r="P221" t="n">
-        <v>1.24</v>
+        <v>1.274</v>
       </c>
       <c r="Q221" t="n">
-        <v>0.573</v>
+        <v>0.585</v>
       </c>
       <c r="R221" t="n">
-        <v>0.455</v>
+        <v>0.489</v>
       </c>
       <c r="S221" t="n">
-        <v>0.158</v>
+        <v>0.155</v>
       </c>
       <c r="T221" t="n">
-        <v>0.013</v>
+        <v>0.008</v>
       </c>
       <c r="U221" t="n">
-        <v>0.177</v>
+        <v>0.184</v>
       </c>
       <c r="V221" t="n">
-        <v>0.569</v>
+        <v>0.582</v>
       </c>
       <c r="W221" t="n">
-        <v>0.6</v>
+        <v>0.599</v>
       </c>
       <c r="X221" t="n">
-        <v>0.1</v>
+        <v>0.103</v>
       </c>
       <c r="Y221" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="Z221" t="n">
-        <v>7.945</v>
+        <v>8.096</v>
       </c>
       <c r="AA221" t="n">
-        <v>10.704</v>
+        <v>10.888</v>
       </c>
       <c r="AB221" t="n">
-        <v>0.166</v>
+        <v>0.17</v>
       </c>
       <c r="AC221" t="n">
-        <v>0.58</v>
+        <v>0.59</v>
       </c>
       <c r="AD221" t="n">
-        <v>0.083</v>
+        <v>0.081</v>
       </c>
     </row>
     <row r="222">
@@ -24379,61 +24379,61 @@
         <v>4</v>
       </c>
       <c r="L222" t="n">
-        <v>4.568</v>
+        <v>4.534</v>
       </c>
       <c r="M222" t="n">
-        <v>4.068</v>
+        <v>4.051</v>
       </c>
       <c r="N222" t="n">
-        <v>1.179</v>
+        <v>1.173</v>
       </c>
       <c r="O222" t="n">
-        <v>2.197</v>
+        <v>2.084</v>
       </c>
       <c r="P222" t="n">
-        <v>0.749</v>
+        <v>0.745</v>
       </c>
       <c r="Q222" t="n">
-        <v>0.403</v>
+        <v>0.369</v>
       </c>
       <c r="R222" t="n">
-        <v>0.66</v>
+        <v>0.698</v>
       </c>
       <c r="S222" t="n">
-        <v>0.258</v>
+        <v>0.247</v>
       </c>
       <c r="T222" t="n">
-        <v>0.022</v>
+        <v>0.021</v>
       </c>
       <c r="U222" t="n">
-        <v>0.238</v>
+        <v>0.207</v>
       </c>
       <c r="V222" t="n">
-        <v>0.712</v>
+        <v>0.6860000000000001</v>
       </c>
       <c r="W222" t="n">
-        <v>0.714</v>
+        <v>0.679</v>
       </c>
       <c r="X222" t="n">
-        <v>0.036</v>
+        <v>0.033</v>
       </c>
       <c r="Y222" t="n">
-        <v>0.03</v>
+        <v>0.026</v>
       </c>
       <c r="Z222" t="n">
-        <v>9.640000000000001</v>
+        <v>9.167</v>
       </c>
       <c r="AA222" t="n">
-        <v>12.755</v>
+        <v>12.088</v>
       </c>
       <c r="AB222" t="n">
-        <v>0.212</v>
+        <v>0.192</v>
       </c>
       <c r="AC222" t="n">
-        <v>0.724</v>
+        <v>0.727</v>
       </c>
       <c r="AD222" t="n">
-        <v>0.029</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="223">
@@ -24487,61 +24487,61 @@
         <v>1</v>
       </c>
       <c r="L223" t="n">
-        <v>4.926</v>
+        <v>4.934</v>
       </c>
       <c r="M223" t="n">
-        <v>4.292</v>
+        <v>4.263</v>
       </c>
       <c r="N223" t="n">
-        <v>1.251</v>
+        <v>1.256</v>
       </c>
       <c r="O223" t="n">
-        <v>1.93</v>
+        <v>1.931</v>
       </c>
       <c r="P223" t="n">
-        <v>0.541</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="Q223" t="n">
-        <v>0.522</v>
+        <v>0.556</v>
       </c>
       <c r="R223" t="n">
-        <v>0.874</v>
+        <v>0.889</v>
       </c>
       <c r="S223" t="n">
-        <v>0.217</v>
+        <v>0.201</v>
       </c>
       <c r="T223" t="n">
-        <v>0.018</v>
+        <v>0.023</v>
       </c>
       <c r="U223" t="n">
-        <v>0.142</v>
+        <v>0.143</v>
       </c>
       <c r="V223" t="n">
-        <v>0.571</v>
+        <v>0.595</v>
       </c>
       <c r="W223" t="n">
-        <v>0.797</v>
+        <v>0.756</v>
       </c>
       <c r="X223" t="n">
-        <v>0.216</v>
+        <v>0.222</v>
       </c>
       <c r="Y223" t="n">
-        <v>0.183</v>
+        <v>0.19</v>
       </c>
       <c r="Z223" t="n">
-        <v>9.965999999999999</v>
+        <v>10.044</v>
       </c>
       <c r="AA223" t="n">
-        <v>13.002</v>
+        <v>13.098</v>
       </c>
       <c r="AB223" t="n">
-        <v>0.135</v>
+        <v>0.133</v>
       </c>
       <c r="AC223" t="n">
-        <v>0.747</v>
+        <v>0.752</v>
       </c>
       <c r="AD223" t="n">
-        <v>0.173</v>
+        <v>0.176</v>
       </c>
     </row>
     <row r="224">
@@ -24595,61 +24595,61 @@
         <v>4</v>
       </c>
       <c r="L224" t="n">
-        <v>4.475</v>
+        <v>4.451</v>
       </c>
       <c r="M224" t="n">
-        <v>3.666</v>
+        <v>3.664</v>
       </c>
       <c r="N224" t="n">
-        <v>0.864</v>
+        <v>0.884</v>
       </c>
       <c r="O224" t="n">
-        <v>1.663</v>
+        <v>1.617</v>
       </c>
       <c r="P224" t="n">
-        <v>1.387</v>
+        <v>1.377</v>
       </c>
       <c r="Q224" t="n">
-        <v>0.726</v>
+        <v>0.706</v>
       </c>
       <c r="R224" t="n">
-        <v>0.486</v>
+        <v>0.519</v>
       </c>
       <c r="S224" t="n">
-        <v>0.162</v>
+        <v>0.175</v>
       </c>
       <c r="T224" t="n">
-        <v>0.013</v>
+        <v>0.012</v>
       </c>
       <c r="U224" t="n">
-        <v>0.203</v>
+        <v>0.178</v>
       </c>
       <c r="V224" t="n">
-        <v>0.715</v>
+        <v>0.664</v>
       </c>
       <c r="W224" t="n">
-        <v>0.675</v>
+        <v>0.635</v>
       </c>
       <c r="X224" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="Y224" t="n">
+        <v>0.054</v>
+      </c>
+      <c r="Z224" t="n">
+        <v>8.586</v>
+      </c>
+      <c r="AA224" t="n">
+        <v>11.646</v>
+      </c>
+      <c r="AB224" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="AC224" t="n">
+        <v>0.611</v>
+      </c>
+      <c r="AD224" t="n">
         <v>0.052</v>
-      </c>
-      <c r="Y224" t="n">
-        <v>0.042</v>
-      </c>
-      <c r="Z224" t="n">
-        <v>8.85</v>
-      </c>
-      <c r="AA224" t="n">
-        <v>12.084</v>
-      </c>
-      <c r="AB224" t="n">
-        <v>0.187</v>
-      </c>
-      <c r="AC224" t="n">
-        <v>0.602</v>
-      </c>
-      <c r="AD224" t="n">
-        <v>0.041</v>
       </c>
     </row>
     <row r="225">
@@ -24703,61 +24703,61 @@
         <v>2</v>
       </c>
       <c r="L225" t="n">
-        <v>4.726</v>
+        <v>4.761</v>
       </c>
       <c r="M225" t="n">
-        <v>4.244</v>
+        <v>4.263</v>
       </c>
       <c r="N225" t="n">
-        <v>1.155</v>
+        <v>1.135</v>
       </c>
       <c r="O225" t="n">
-        <v>2.211</v>
+        <v>2.15</v>
       </c>
       <c r="P225" t="n">
-        <v>1.047</v>
+        <v>1.068</v>
       </c>
       <c r="Q225" t="n">
         <v>0.386</v>
       </c>
       <c r="R225" t="n">
-        <v>0.627</v>
+        <v>0.632</v>
       </c>
       <c r="S225" t="n">
-        <v>0.257</v>
+        <v>0.239</v>
       </c>
       <c r="T225" t="n">
-        <v>0.014</v>
+        <v>0.017</v>
       </c>
       <c r="U225" t="n">
-        <v>0.257</v>
+        <v>0.247</v>
       </c>
       <c r="V225" t="n">
-        <v>0.679</v>
+        <v>0.657</v>
       </c>
       <c r="W225" t="n">
-        <v>0.746</v>
+        <v>0.727</v>
       </c>
       <c r="X225" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Y225" t="n">
         <v>0.042</v>
       </c>
-      <c r="Y225" t="n">
-        <v>0.035</v>
-      </c>
       <c r="Z225" t="n">
-        <v>9.643000000000001</v>
+        <v>9.446</v>
       </c>
       <c r="AA225" t="n">
-        <v>12.763</v>
+        <v>12.482</v>
       </c>
       <c r="AB225" t="n">
-        <v>0.224</v>
+        <v>0.222</v>
       </c>
       <c r="AC225" t="n">
-        <v>0.719</v>
+        <v>0.714</v>
       </c>
       <c r="AD225" t="n">
-        <v>0.034</v>
+        <v>0.041</v>
       </c>
     </row>
     <row r="226">
@@ -24811,61 +24811,61 @@
         <v>1</v>
       </c>
       <c r="L226" t="n">
-        <v>4.81</v>
+        <v>4.834</v>
       </c>
       <c r="M226" t="n">
-        <v>4.269</v>
+        <v>4.283</v>
       </c>
       <c r="N226" t="n">
-        <v>1.058</v>
+        <v>1.05</v>
       </c>
       <c r="O226" t="n">
-        <v>2.095</v>
+        <v>1.992</v>
       </c>
       <c r="P226" t="n">
-        <v>1.279</v>
+        <v>1.302</v>
       </c>
       <c r="Q226" t="n">
-        <v>0.437</v>
+        <v>0.447</v>
       </c>
       <c r="R226" t="n">
-        <v>0.544</v>
+        <v>0.58</v>
       </c>
       <c r="S226" t="n">
-        <v>0.24</v>
+        <v>0.223</v>
       </c>
       <c r="T226" t="n">
-        <v>0.026</v>
+        <v>0.022</v>
       </c>
       <c r="U226" t="n">
-        <v>0.248</v>
+        <v>0.225</v>
       </c>
       <c r="V226" t="n">
-        <v>0.609</v>
+        <v>0.547</v>
       </c>
       <c r="W226" t="n">
-        <v>0.751</v>
+        <v>0.744</v>
       </c>
       <c r="X226" t="n">
-        <v>0.298</v>
+        <v>0.294</v>
       </c>
       <c r="Y226" t="n">
-        <v>0.252</v>
+        <v>0.241</v>
       </c>
       <c r="Z226" t="n">
-        <v>10.38</v>
+        <v>9.962999999999999</v>
       </c>
       <c r="AA226" t="n">
-        <v>13.647</v>
+        <v>13.059</v>
       </c>
       <c r="AB226" t="n">
-        <v>0.223</v>
+        <v>0.205</v>
       </c>
       <c r="AC226" t="n">
         <v>0.6820000000000001</v>
       </c>
       <c r="AD226" t="n">
-        <v>0.225</v>
+        <v>0.217</v>
       </c>
     </row>
     <row r="227">
@@ -24919,61 +24919,61 @@
         <v>3</v>
       </c>
       <c r="L227" t="n">
-        <v>4.563</v>
+        <v>4.573</v>
       </c>
       <c r="M227" t="n">
         <v>4.03</v>
       </c>
       <c r="N227" t="n">
-        <v>1.03</v>
+        <v>1.072</v>
       </c>
       <c r="O227" t="n">
-        <v>1.903</v>
+        <v>1.881</v>
       </c>
       <c r="P227" t="n">
-        <v>1.023</v>
+        <v>0.974</v>
       </c>
       <c r="Q227" t="n">
-        <v>0.434</v>
+        <v>0.446</v>
       </c>
       <c r="R227" t="n">
-        <v>0.5659999999999999</v>
+        <v>0.641</v>
       </c>
       <c r="S227" t="n">
-        <v>0.244</v>
+        <v>0.227</v>
       </c>
       <c r="T227" t="n">
-        <v>0.03</v>
+        <v>0.031</v>
       </c>
       <c r="U227" t="n">
-        <v>0.189</v>
+        <v>0.173</v>
       </c>
       <c r="V227" t="n">
-        <v>0.615</v>
+        <v>0.581</v>
       </c>
       <c r="W227" t="n">
-        <v>0.643</v>
+        <v>0.639</v>
       </c>
       <c r="X227" t="n">
-        <v>0.044</v>
+        <v>0.052</v>
       </c>
       <c r="Y227" t="n">
-        <v>0.036</v>
+        <v>0.043</v>
       </c>
       <c r="Z227" t="n">
-        <v>8.619999999999999</v>
+        <v>8.585000000000001</v>
       </c>
       <c r="AA227" t="n">
-        <v>11.438</v>
+        <v>11.317</v>
       </c>
       <c r="AB227" t="n">
-        <v>0.178</v>
+        <v>0.161</v>
       </c>
       <c r="AC227" t="n">
-        <v>0.675</v>
+        <v>0.6870000000000001</v>
       </c>
       <c r="AD227" t="n">
-        <v>0.036</v>
+        <v>0.042</v>
       </c>
     </row>
     <row r="228">
@@ -25027,61 +25027,61 @@
         <v>5</v>
       </c>
       <c r="L228" t="n">
-        <v>4.401</v>
+        <v>4.406</v>
       </c>
       <c r="M228" t="n">
-        <v>3.576</v>
+        <v>3.569</v>
       </c>
       <c r="N228" t="n">
-        <v>0.883</v>
+        <v>0.905</v>
       </c>
       <c r="O228" t="n">
-        <v>1.683</v>
+        <v>1.684</v>
       </c>
       <c r="P228" t="n">
-        <v>1.247</v>
+        <v>1.222</v>
       </c>
       <c r="Q228" t="n">
         <v>0.737</v>
       </c>
       <c r="R228" t="n">
-        <v>0.488</v>
+        <v>0.517</v>
       </c>
       <c r="S228" t="n">
         <v>0.18</v>
       </c>
       <c r="T228" t="n">
-        <v>0.027</v>
+        <v>0.024</v>
       </c>
       <c r="U228" t="n">
-        <v>0.189</v>
+        <v>0.184</v>
       </c>
       <c r="V228" t="n">
-        <v>0.717</v>
+        <v>0.702</v>
       </c>
       <c r="W228" t="n">
-        <v>0.673</v>
+        <v>0.677</v>
       </c>
       <c r="X228" t="n">
-        <v>0.076</v>
+        <v>0.081</v>
       </c>
       <c r="Y228" t="n">
-        <v>0.062</v>
+        <v>0.067</v>
       </c>
       <c r="Z228" t="n">
-        <v>9.029</v>
+        <v>9.045</v>
       </c>
       <c r="AA228" t="n">
-        <v>12.295</v>
+        <v>12.285</v>
       </c>
       <c r="AB228" t="n">
-        <v>0.175</v>
+        <v>0.171</v>
       </c>
       <c r="AC228" t="n">
-        <v>0.618</v>
+        <v>0.628</v>
       </c>
       <c r="AD228" t="n">
-        <v>0.061</v>
+        <v>0.065</v>
       </c>
     </row>
     <row r="229">
@@ -25135,61 +25135,61 @@
         <v>9</v>
       </c>
       <c r="L229" t="n">
-        <v>3.852</v>
+        <v>3.837</v>
       </c>
       <c r="M229" t="n">
-        <v>3.481</v>
+        <v>3.437</v>
       </c>
       <c r="N229" t="n">
-        <v>0.842</v>
+        <v>0.827</v>
       </c>
       <c r="O229" t="n">
-        <v>1.605</v>
+        <v>1.553</v>
       </c>
       <c r="P229" t="n">
-        <v>1.052</v>
+        <v>0.993</v>
       </c>
       <c r="Q229" t="n">
-        <v>0.295</v>
+        <v>0.318</v>
       </c>
       <c r="R229" t="n">
-        <v>0.433</v>
+        <v>0.441</v>
       </c>
       <c r="S229" t="n">
-        <v>0.232</v>
+        <v>0.216</v>
       </c>
       <c r="T229" t="n">
         <v>0</v>
       </c>
       <c r="U229" t="n">
-        <v>0.177</v>
+        <v>0.17</v>
       </c>
       <c r="V229" t="n">
-        <v>0.547</v>
+        <v>0.523</v>
       </c>
       <c r="W229" t="n">
-        <v>0.535</v>
+        <v>0.505</v>
       </c>
       <c r="X229" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="Y229" t="n">
         <v>0.034</v>
       </c>
-      <c r="Y229" t="n">
-        <v>0.03</v>
-      </c>
       <c r="Z229" t="n">
-        <v>7.133</v>
+        <v>6.965</v>
       </c>
       <c r="AA229" t="n">
-        <v>9.507</v>
+        <v>9.263</v>
       </c>
       <c r="AB229" t="n">
-        <v>0.166</v>
+        <v>0.154</v>
       </c>
       <c r="AC229" t="n">
-        <v>0.597</v>
+        <v>0.581</v>
       </c>
       <c r="AD229" t="n">
-        <v>0.029</v>
+        <v>0.033</v>
       </c>
     </row>
     <row r="230">
@@ -25207,16 +25207,16 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>683737</v>
+        <v>687462</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Michael Busch</t>
+          <t>Spencer Horwitz</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>Busch</t>
+          <t>Horwitz</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
@@ -25226,78 +25226,78 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
         <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
           <t>CHC</t>
         </is>
       </c>
-      <c r="J230" t="inlineStr">
-        <is>
-          <t>PIT</t>
-        </is>
-      </c>
       <c r="K230" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L230" t="n">
-        <v>4.659</v>
+        <v>4.32</v>
       </c>
       <c r="M230" t="n">
-        <v>3.854</v>
+        <v>3.757</v>
       </c>
       <c r="N230" t="n">
-        <v>1.119</v>
+        <v>1.064</v>
       </c>
       <c r="O230" t="n">
-        <v>2.187</v>
+        <v>1.916</v>
       </c>
       <c r="P230" t="n">
-        <v>1.1</v>
+        <v>0.66</v>
       </c>
       <c r="Q230" t="n">
-        <v>0.724</v>
+        <v>0.464</v>
       </c>
       <c r="R230" t="n">
-        <v>0.612</v>
+        <v>0.615</v>
       </c>
       <c r="S230" t="n">
-        <v>0.218</v>
+        <v>0.248</v>
       </c>
       <c r="T230" t="n">
-        <v>0.019</v>
+        <v>0</v>
       </c>
       <c r="U230" t="n">
-        <v>0.271</v>
+        <v>0.201</v>
       </c>
       <c r="V230" t="n">
-        <v>0.756</v>
+        <v>0.661</v>
       </c>
       <c r="W230" t="n">
-        <v>0.825</v>
+        <v>0.6</v>
       </c>
       <c r="X230" t="n">
-        <v>0.037</v>
+        <v>0.026</v>
       </c>
       <c r="Y230" t="n">
-        <v>0.03</v>
+        <v>0.021</v>
       </c>
       <c r="Z230" t="n">
-        <v>10.54</v>
+        <v>8.656000000000001</v>
       </c>
       <c r="AA230" t="n">
-        <v>14.196</v>
+        <v>11.505</v>
       </c>
       <c r="AB230" t="n">
-        <v>0.241</v>
+        <v>0.186</v>
       </c>
       <c r="AC230" t="n">
-        <v>0.709</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="AD230" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="231">
@@ -25315,16 +25315,16 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>687462</v>
+        <v>691718</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Spencer Horwitz</t>
+          <t>Pete Crow-Armstrong</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>Horwitz</t>
+          <t>Crow-Armstrong</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
@@ -25334,78 +25334,78 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
         <is>
+          <t>CHC</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
           <t>PIT</t>
-        </is>
-      </c>
-      <c r="J231" t="inlineStr">
-        <is>
-          <t>CHC</t>
         </is>
       </c>
       <c r="K231" t="n">
         <v>7</v>
       </c>
       <c r="L231" t="n">
-        <v>4.33</v>
+        <v>4.183</v>
       </c>
       <c r="M231" t="n">
-        <v>3.776</v>
+        <v>3.786</v>
       </c>
       <c r="N231" t="n">
-        <v>1.063</v>
+        <v>0.948</v>
       </c>
       <c r="O231" t="n">
-        <v>1.889</v>
+        <v>1.706</v>
       </c>
       <c r="P231" t="n">
-        <v>0.662</v>
+        <v>1.194</v>
       </c>
       <c r="Q231" t="n">
-        <v>0.457</v>
+        <v>0.303</v>
       </c>
       <c r="R231" t="n">
-        <v>0.616</v>
+        <v>0.554</v>
       </c>
       <c r="S231" t="n">
-        <v>0.257</v>
+        <v>0.198</v>
       </c>
       <c r="T231" t="n">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="U231" t="n">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
       <c r="V231" t="n">
-        <v>0.64</v>
+        <v>0.639</v>
       </c>
       <c r="W231" t="n">
-        <v>0.624</v>
+        <v>0.55</v>
       </c>
       <c r="X231" t="n">
-        <v>0.026</v>
+        <v>0.286</v>
       </c>
       <c r="Y231" t="n">
-        <v>0.021</v>
+        <v>0.232</v>
       </c>
       <c r="Z231" t="n">
-        <v>8.577</v>
+        <v>8.699</v>
       </c>
       <c r="AA231" t="n">
-        <v>11.4</v>
+        <v>11.416</v>
       </c>
       <c r="AB231" t="n">
-        <v>0.174</v>
+        <v>0.158</v>
       </c>
       <c r="AC231" t="n">
-        <v>0.677</v>
+        <v>0.642</v>
       </c>
       <c r="AD231" t="n">
-        <v>0.021</v>
+        <v>0.209</v>
       </c>
     </row>
     <row r="232">
@@ -25423,97 +25423,97 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>691718</v>
+        <v>693304</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Pete Crow-Armstrong</t>
+          <t>Nick Gonzales</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>Crow-Armstrong</t>
+          <t>Gonzales</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
         <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
           <t>CHC</t>
-        </is>
-      </c>
-      <c r="J232" t="inlineStr">
-        <is>
-          <t>PIT</t>
         </is>
       </c>
       <c r="K232" t="n">
         <v>6</v>
       </c>
       <c r="L232" t="n">
-        <v>4.303</v>
+        <v>4.338</v>
       </c>
       <c r="M232" t="n">
-        <v>3.895</v>
+        <v>4.034</v>
       </c>
       <c r="N232" t="n">
-        <v>1.007</v>
+        <v>1.163</v>
       </c>
       <c r="O232" t="n">
-        <v>1.882</v>
+        <v>1.883</v>
       </c>
       <c r="P232" t="n">
-        <v>1.211</v>
+        <v>0.644</v>
       </c>
       <c r="Q232" t="n">
-        <v>0.324</v>
+        <v>0.196</v>
       </c>
       <c r="R232" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.744</v>
       </c>
       <c r="S232" t="n">
-        <v>0.217</v>
+        <v>0.257</v>
       </c>
       <c r="T232" t="n">
-        <v>0.029</v>
+        <v>0.025</v>
       </c>
       <c r="U232" t="n">
-        <v>0.2</v>
+        <v>0.138</v>
       </c>
       <c r="V232" t="n">
-        <v>0.753</v>
+        <v>0.58</v>
       </c>
       <c r="W232" t="n">
-        <v>0.624</v>
+        <v>0.577</v>
       </c>
       <c r="X232" t="n">
-        <v>0.309</v>
+        <v>0.041</v>
       </c>
       <c r="Y232" t="n">
-        <v>0.255</v>
+        <v>0.034</v>
       </c>
       <c r="Z232" t="n">
-        <v>9.677</v>
+        <v>7.966</v>
       </c>
       <c r="AA232" t="n">
-        <v>12.781</v>
+        <v>10.316</v>
       </c>
       <c r="AB232" t="n">
-        <v>0.182</v>
+        <v>0.13</v>
       </c>
       <c r="AC232" t="n">
-        <v>0.667</v>
+        <v>0.713</v>
       </c>
       <c r="AD232" t="n">
-        <v>0.228</v>
+        <v>0.033</v>
       </c>
     </row>
     <row r="233">
@@ -25531,97 +25531,97 @@
         </is>
       </c>
       <c r="D233" t="n">
-        <v>693304</v>
+        <v>694208</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Nick Gonzales</t>
+          <t>Moises Ballesteros</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>Gonzales</t>
+          <t>Ballesteros</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
         <is>
+          <t>CHC</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
           <t>PIT</t>
         </is>
       </c>
-      <c r="J233" t="inlineStr">
-        <is>
-          <t>CHC</t>
-        </is>
-      </c>
       <c r="K233" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L233" t="n">
-        <v>4.337</v>
+        <v>4.596</v>
       </c>
       <c r="M233" t="n">
-        <v>4.023</v>
+        <v>3.936</v>
       </c>
       <c r="N233" t="n">
-        <v>1.168</v>
+        <v>0.964</v>
       </c>
       <c r="O233" t="n">
-        <v>1.888</v>
+        <v>1.657</v>
       </c>
       <c r="P233" t="n">
+        <v>1.264</v>
+      </c>
+      <c r="Q233" t="n">
+        <v>0.5639999999999999</v>
+      </c>
+      <c r="R233" t="n">
+        <v>0.611</v>
+      </c>
+      <c r="S233" t="n">
+        <v>0.177</v>
+      </c>
+      <c r="T233" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="U233" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="V233" t="n">
+        <v>0.571</v>
+      </c>
+      <c r="W233" t="n">
         <v>0.637</v>
       </c>
-      <c r="Q233" t="n">
-        <v>0.206</v>
-      </c>
-      <c r="R233" t="n">
-        <v>0.738</v>
-      </c>
-      <c r="S233" t="n">
-        <v>0.275</v>
-      </c>
-      <c r="T233" t="n">
-        <v>0.022</v>
-      </c>
-      <c r="U233" t="n">
-        <v>0.134</v>
-      </c>
-      <c r="V233" t="n">
-        <v>0.584</v>
-      </c>
-      <c r="W233" t="n">
-        <v>0.587</v>
-      </c>
       <c r="X233" t="n">
-        <v>0.038</v>
+        <v>0.033</v>
       </c>
       <c r="Y233" t="n">
-        <v>0.031</v>
+        <v>0.027</v>
       </c>
       <c r="Z233" t="n">
-        <v>8.007</v>
+        <v>8.132999999999999</v>
       </c>
       <c r="AA233" t="n">
-        <v>10.388</v>
+        <v>10.862</v>
       </c>
       <c r="AB233" t="n">
-        <v>0.126</v>
+        <v>0.153</v>
       </c>
       <c r="AC233" t="n">
-        <v>0.714</v>
+        <v>0.637</v>
       </c>
       <c r="AD233" t="n">
-        <v>0.031</v>
+        <v>0.027</v>
       </c>
     </row>
     <row r="234">
@@ -25639,97 +25639,97 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>694208</v>
+        <v>804606</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Moises Ballesteros</t>
+          <t>Konnor Griffin</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>Ballesteros</t>
+          <t>Griffin</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I234" t="inlineStr">
         <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
           <t>CHC</t>
-        </is>
-      </c>
-      <c r="J234" t="inlineStr">
-        <is>
-          <t>PIT</t>
         </is>
       </c>
       <c r="K234" t="n">
         <v>8</v>
       </c>
       <c r="L234" t="n">
-        <v>4.018</v>
+        <v>4.088</v>
       </c>
       <c r="M234" t="n">
-        <v>3.465</v>
+        <v>3.755</v>
       </c>
       <c r="N234" t="n">
-        <v>0.84</v>
+        <v>0.854</v>
       </c>
       <c r="O234" t="n">
-        <v>1.491</v>
+        <v>1.464</v>
       </c>
       <c r="P234" t="n">
-        <v>1.111</v>
+        <v>0.991</v>
       </c>
       <c r="Q234" t="n">
-        <v>0.482</v>
+        <v>0.248</v>
       </c>
       <c r="R234" t="n">
-        <v>0.515</v>
+        <v>0.524</v>
       </c>
       <c r="S234" t="n">
-        <v>0.156</v>
+        <v>0.191</v>
       </c>
       <c r="T234" t="n">
-        <v>0.008999999999999999</v>
+        <v>0</v>
       </c>
       <c r="U234" t="n">
-        <v>0.159</v>
+        <v>0.14</v>
       </c>
       <c r="V234" t="n">
-        <v>0.549</v>
+        <v>0.503</v>
       </c>
       <c r="W234" t="n">
-        <v>0.582</v>
+        <v>0.473</v>
       </c>
       <c r="X234" t="n">
-        <v>0.022</v>
+        <v>0.134</v>
       </c>
       <c r="Y234" t="n">
-        <v>0.018</v>
+        <v>0.113</v>
       </c>
       <c r="Z234" t="n">
-        <v>7.305</v>
+        <v>6.932</v>
       </c>
       <c r="AA234" t="n">
-        <v>9.81</v>
+        <v>9.084</v>
       </c>
       <c r="AB234" t="n">
-        <v>0.147</v>
+        <v>0.132</v>
       </c>
       <c r="AC234" t="n">
-        <v>0.579</v>
+        <v>0.594</v>
       </c>
       <c r="AD234" t="n">
-        <v>0.017</v>
+        <v>0.107</v>
       </c>
     </row>
     <row r="235">
@@ -25747,16 +25747,16 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>804606</v>
+        <v>807713</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Konnor Griffin</t>
+          <t>Matt Shaw</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>Griffin</t>
+          <t>Shaw</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
@@ -25766,78 +25766,78 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
         <is>
+          <t>CHC</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
           <t>PIT</t>
         </is>
       </c>
-      <c r="J235" t="inlineStr">
-        <is>
-          <t>CHC</t>
-        </is>
-      </c>
       <c r="K235" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L235" t="n">
-        <v>4.131</v>
+        <v>3.766</v>
       </c>
       <c r="M235" t="n">
-        <v>3.789</v>
+        <v>3.172</v>
       </c>
       <c r="N235" t="n">
-        <v>0.906</v>
+        <v>0.779</v>
       </c>
       <c r="O235" t="n">
-        <v>1.607</v>
+        <v>1.269</v>
       </c>
       <c r="P235" t="n">
-        <v>0.995</v>
+        <v>0.959</v>
       </c>
       <c r="Q235" t="n">
-        <v>0.253</v>
+        <v>0.516</v>
       </c>
       <c r="R235" t="n">
-        <v>0.537</v>
+        <v>0.497</v>
       </c>
       <c r="S235" t="n">
-        <v>0.202</v>
+        <v>0.175</v>
       </c>
       <c r="T235" t="n">
-        <v>0</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="U235" t="n">
-        <v>0.166</v>
+        <v>0.099</v>
       </c>
       <c r="V235" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.441</v>
       </c>
       <c r="W235" t="n">
-        <v>0.529</v>
+        <v>0.521</v>
       </c>
       <c r="X235" t="n">
-        <v>0.142</v>
+        <v>0.146</v>
       </c>
       <c r="Y235" t="n">
-        <v>0.114</v>
+        <v>0.121</v>
       </c>
       <c r="Z235" t="n">
-        <v>7.54</v>
+        <v>6.986</v>
       </c>
       <c r="AA235" t="n">
-        <v>9.917</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="AB235" t="n">
-        <v>0.156</v>
+        <v>0.095</v>
       </c>
       <c r="AC235" t="n">
-        <v>0.617</v>
+        <v>0.5629999999999999</v>
       </c>
       <c r="AD235" t="n">
-        <v>0.11</v>
+        <v>0.115</v>
       </c>
     </row>
     <row r="236">

</xml_diff>

<commit_message>
feat: slate size auto-detection, constraint relaxation, dashboard warnings — Codex implementation
</commit_message>
<xml_diff>
--- a/data/live/BallparkPal_Batters_2026-04-12.xlsx
+++ b/data/live/BallparkPal_Batters_2026-04-12.xlsx
@@ -8355,16 +8355,16 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>592518</v>
+        <v>592206</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Manny Machado</t>
+          <t>Nick Castellanos</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Machado</t>
+          <t>Castellanos</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -8388,64 +8388,64 @@
         </is>
       </c>
       <c r="K74" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L74" t="n">
-        <v>4.25</v>
+        <v>3.903</v>
       </c>
       <c r="M74" t="n">
-        <v>3.743</v>
+        <v>3.617</v>
       </c>
       <c r="N74" t="n">
-        <v>1.02</v>
+        <v>0.843</v>
       </c>
       <c r="O74" t="n">
-        <v>1.71</v>
+        <v>1.371</v>
       </c>
       <c r="P74" t="n">
-        <v>0.862</v>
+        <v>0.905</v>
       </c>
       <c r="Q74" t="n">
-        <v>0.412</v>
+        <v>0.195</v>
       </c>
       <c r="R74" t="n">
-        <v>0.673</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="S74" t="n">
-        <v>0.172</v>
+        <v>0.149</v>
       </c>
       <c r="T74" t="n">
-        <v>0.007</v>
+        <v>0.015</v>
       </c>
       <c r="U74" t="n">
-        <v>0.168</v>
+        <v>0.116</v>
       </c>
       <c r="V74" t="n">
-        <v>0.61</v>
+        <v>0.462</v>
       </c>
       <c r="W74" t="n">
-        <v>0.5679999999999999</v>
+        <v>0.403</v>
       </c>
       <c r="X74" t="n">
-        <v>0.083</v>
+        <v>0.041</v>
       </c>
       <c r="Y74" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.034</v>
       </c>
       <c r="Z74" t="n">
-        <v>8.140000000000001</v>
+        <v>6.006</v>
       </c>
       <c r="AA74" t="n">
-        <v>10.734</v>
+        <v>7.809</v>
       </c>
       <c r="AB74" t="n">
-        <v>0.157</v>
+        <v>0.11</v>
       </c>
       <c r="AC74" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.596</v>
       </c>
       <c r="AD74" t="n">
-        <v>0.067</v>
+        <v>0.034</v>
       </c>
     </row>
     <row r="75">
@@ -8463,16 +8463,16 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>593428</v>
+        <v>592518</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Xander Bogaerts</t>
+          <t>Manny Machado</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Bogaerts</t>
+          <t>Machado</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -8496,64 +8496,64 @@
         </is>
       </c>
       <c r="K75" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L75" t="n">
-        <v>3.966</v>
+        <v>4.25</v>
       </c>
       <c r="M75" t="n">
-        <v>3.55</v>
+        <v>3.733</v>
       </c>
       <c r="N75" t="n">
-        <v>0.902</v>
+        <v>0.994</v>
       </c>
       <c r="O75" t="n">
-        <v>1.34</v>
+        <v>1.676</v>
       </c>
       <c r="P75" t="n">
-        <v>0.547</v>
+        <v>0.874</v>
       </c>
       <c r="Q75" t="n">
-        <v>0.328</v>
+        <v>0.424</v>
       </c>
       <c r="R75" t="n">
-        <v>0.658</v>
+        <v>0.655</v>
       </c>
       <c r="S75" t="n">
-        <v>0.143</v>
+        <v>0.164</v>
       </c>
       <c r="T75" t="n">
         <v>0.008</v>
       </c>
       <c r="U75" t="n">
-        <v>0.093</v>
+        <v>0.167</v>
       </c>
       <c r="V75" t="n">
-        <v>0.449</v>
+        <v>0.591</v>
       </c>
       <c r="W75" t="n">
-        <v>0.442</v>
+        <v>0.536</v>
       </c>
       <c r="X75" t="n">
-        <v>0.117</v>
+        <v>0.079</v>
       </c>
       <c r="Y75" t="n">
-        <v>0.095</v>
+        <v>0.064</v>
       </c>
       <c r="Z75" t="n">
-        <v>6.597</v>
+        <v>7.947</v>
       </c>
       <c r="AA75" t="n">
-        <v>8.561</v>
+        <v>10.472</v>
       </c>
       <c r="AB75" t="n">
-        <v>0.089</v>
+        <v>0.156</v>
       </c>
       <c r="AC75" t="n">
-        <v>0.622</v>
+        <v>0.669</v>
       </c>
       <c r="AD75" t="n">
-        <v>0.092</v>
+        <v>0.063</v>
       </c>
     </row>
     <row r="76">
@@ -8571,16 +8571,16 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>609280</v>
+        <v>593428</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Miguel Andujar</t>
+          <t>Xander Bogaerts</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Andujar</t>
+          <t>Bogaerts</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -8607,61 +8607,61 @@
         <v>5</v>
       </c>
       <c r="L76" t="n">
-        <v>4.055</v>
+        <v>4.042</v>
       </c>
       <c r="M76" t="n">
-        <v>3.717</v>
+        <v>3.615</v>
       </c>
       <c r="N76" t="n">
-        <v>1.029</v>
+        <v>0.883</v>
       </c>
       <c r="O76" t="n">
-        <v>1.436</v>
+        <v>1.335</v>
       </c>
       <c r="P76" t="n">
-        <v>0.589</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="Q76" t="n">
-        <v>0.233</v>
+        <v>0.335</v>
       </c>
       <c r="R76" t="n">
-        <v>0.783</v>
+        <v>0.635</v>
       </c>
       <c r="S76" t="n">
-        <v>0.16</v>
+        <v>0.144</v>
       </c>
       <c r="T76" t="n">
-        <v>0.011</v>
+        <v>0.004</v>
       </c>
       <c r="U76" t="n">
-        <v>0.075</v>
+        <v>0.1</v>
       </c>
       <c r="V76" t="n">
-        <v>0.447</v>
+        <v>0.454</v>
       </c>
       <c r="W76" t="n">
-        <v>0.457</v>
+        <v>0.451</v>
       </c>
       <c r="X76" t="n">
-        <v>0.044</v>
+        <v>0.1</v>
       </c>
       <c r="Y76" t="n">
-        <v>0.034</v>
+        <v>0.081</v>
       </c>
       <c r="Z76" t="n">
-        <v>6.431</v>
+        <v>6.543</v>
       </c>
       <c r="AA76" t="n">
-        <v>8.237</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="AB76" t="n">
-        <v>0.074</v>
+        <v>0.095</v>
       </c>
       <c r="AC76" t="n">
-        <v>0.681</v>
+        <v>0.619</v>
       </c>
       <c r="AD76" t="n">
-        <v>0.032</v>
+        <v>0.076</v>
       </c>
     </row>
     <row r="77">
@@ -8679,21 +8679,21 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>630105</v>
+        <v>657656</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Jake Cronenworth</t>
+          <t>Ramon Laureano</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Cronenworth</t>
+          <t>Laureano</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -8712,64 +8712,64 @@
         </is>
       </c>
       <c r="K77" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L77" t="n">
-        <v>3.687</v>
+        <v>4.51</v>
       </c>
       <c r="M77" t="n">
-        <v>3.171</v>
+        <v>4.024</v>
       </c>
       <c r="N77" t="n">
-        <v>0.792</v>
+        <v>1.035</v>
       </c>
       <c r="O77" t="n">
-        <v>1.191</v>
+        <v>1.747</v>
       </c>
       <c r="P77" t="n">
-        <v>0.731</v>
+        <v>0.944</v>
       </c>
       <c r="Q77" t="n">
-        <v>0.429</v>
+        <v>0.376</v>
       </c>
       <c r="R77" t="n">
-        <v>0.571</v>
+        <v>0.676</v>
       </c>
       <c r="S77" t="n">
-        <v>0.12</v>
+        <v>0.177</v>
       </c>
       <c r="T77" t="n">
-        <v>0.021</v>
+        <v>0.012</v>
       </c>
       <c r="U77" t="n">
-        <v>0.079</v>
+        <v>0.17</v>
       </c>
       <c r="V77" t="n">
-        <v>0.393</v>
+        <v>0.488</v>
       </c>
       <c r="W77" t="n">
-        <v>0.432</v>
+        <v>0.631</v>
       </c>
       <c r="X77" t="n">
-        <v>0.033</v>
+        <v>0.18</v>
       </c>
       <c r="Y77" t="n">
-        <v>0.025</v>
+        <v>0.147</v>
       </c>
       <c r="Z77" t="n">
-        <v>5.908</v>
+        <v>8.438000000000001</v>
       </c>
       <c r="AA77" t="n">
-        <v>7.769</v>
+        <v>10.98</v>
       </c>
       <c r="AB77" t="n">
-        <v>0.077</v>
+        <v>0.159</v>
       </c>
       <c r="AC77" t="n">
-        <v>0.581</v>
+        <v>0.668</v>
       </c>
       <c r="AD77" t="n">
-        <v>0.025</v>
+        <v>0.137</v>
       </c>
     </row>
     <row r="78">
@@ -8787,97 +8787,97 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>650489</v>
+        <v>664034</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Willi Castro</t>
+          <t>Ty France</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Castro</t>
+          <t>France</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>R</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
+          <t xml:space="preserve">SD </t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
           <t>COL</t>
-        </is>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SD </t>
         </is>
       </c>
       <c r="K78" t="n">
         <v>7</v>
       </c>
       <c r="L78" t="n">
-        <v>3.809</v>
+        <v>3.885</v>
       </c>
       <c r="M78" t="n">
-        <v>3.409</v>
+        <v>3.518</v>
       </c>
       <c r="N78" t="n">
-        <v>0.601</v>
+        <v>0.92</v>
       </c>
       <c r="O78" t="n">
-        <v>0.977</v>
+        <v>1.372</v>
       </c>
       <c r="P78" t="n">
-        <v>1.32</v>
+        <v>0.649</v>
       </c>
       <c r="Q78" t="n">
-        <v>0.322</v>
+        <v>0.268</v>
       </c>
       <c r="R78" t="n">
-        <v>0.413</v>
+        <v>0.671</v>
       </c>
       <c r="S78" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.145</v>
       </c>
       <c r="T78" t="n">
-        <v>0.016</v>
+        <v>0.007</v>
       </c>
       <c r="U78" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.098</v>
       </c>
       <c r="V78" t="n">
-        <v>0.266</v>
+        <v>0.431</v>
       </c>
       <c r="W78" t="n">
-        <v>0.285</v>
+        <v>0.415</v>
       </c>
       <c r="X78" t="n">
-        <v>0.113</v>
+        <v>0.023</v>
       </c>
       <c r="Y78" t="n">
-        <v>0.094</v>
+        <v>0.018</v>
       </c>
       <c r="Z78" t="n">
-        <v>4.875</v>
+        <v>6.087</v>
       </c>
       <c r="AA78" t="n">
-        <v>6.306</v>
+        <v>7.866</v>
       </c>
       <c r="AB78" t="n">
-        <v>0.079</v>
+        <v>0.096</v>
       </c>
       <c r="AC78" t="n">
-        <v>0.458</v>
+        <v>0.639</v>
       </c>
       <c r="AD78" t="n">
-        <v>0.089</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="79">
@@ -8895,97 +8895,97 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>657656</v>
+        <v>664954</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Ramon Laureano</t>
+          <t>Brett Sullivan</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Laureano</t>
+          <t>Sullivan</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
           <t xml:space="preserve">SD </t>
         </is>
       </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>COL</t>
-        </is>
-      </c>
       <c r="K79" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L79" t="n">
-        <v>4.51</v>
+        <v>3.614</v>
       </c>
       <c r="M79" t="n">
-        <v>4.045</v>
+        <v>3.348</v>
       </c>
       <c r="N79" t="n">
-        <v>1.021</v>
+        <v>0.611</v>
       </c>
       <c r="O79" t="n">
-        <v>1.705</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="P79" t="n">
-        <v>0.988</v>
+        <v>0.979</v>
       </c>
       <c r="Q79" t="n">
-        <v>0.373</v>
+        <v>0.191</v>
       </c>
       <c r="R79" t="n">
-        <v>0.676</v>
+        <v>0.434</v>
       </c>
       <c r="S79" t="n">
-        <v>0.172</v>
+        <v>0.104</v>
       </c>
       <c r="T79" t="n">
-        <v>0.008</v>
+        <v>0</v>
       </c>
       <c r="U79" t="n">
-        <v>0.166</v>
+        <v>0.073</v>
       </c>
       <c r="V79" t="n">
-        <v>0.496</v>
+        <v>0.254</v>
       </c>
       <c r="W79" t="n">
-        <v>0.62</v>
+        <v>0.256</v>
       </c>
       <c r="X79" t="n">
-        <v>0.179</v>
+        <v>0.018</v>
       </c>
       <c r="Y79" t="n">
-        <v>0.149</v>
+        <v>0.015</v>
       </c>
       <c r="Z79" t="n">
-        <v>8.326000000000001</v>
+        <v>4.029</v>
       </c>
       <c r="AA79" t="n">
-        <v>10.847</v>
+        <v>5.173</v>
       </c>
       <c r="AB79" t="n">
-        <v>0.154</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="AC79" t="n">
-        <v>0.677</v>
+        <v>0.475</v>
       </c>
       <c r="AD79" t="n">
-        <v>0.141</v>
+        <v>0.015</v>
       </c>
     </row>
     <row r="80">
@@ -9003,16 +9003,16 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>664034</v>
+        <v>665487</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Ty France</t>
+          <t>Fernando Tatis Jr.</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Tatis Jr.</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -9036,64 +9036,64 @@
         </is>
       </c>
       <c r="K80" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L80" t="n">
-        <v>3.914</v>
+        <v>4.314</v>
       </c>
       <c r="M80" t="n">
-        <v>3.534</v>
+        <v>3.764</v>
       </c>
       <c r="N80" t="n">
-        <v>0.953</v>
+        <v>0.917</v>
       </c>
       <c r="O80" t="n">
-        <v>1.423</v>
+        <v>1.53</v>
       </c>
       <c r="P80" t="n">
-        <v>0.621</v>
+        <v>1.004</v>
       </c>
       <c r="Q80" t="n">
-        <v>0.3</v>
+        <v>0.45</v>
       </c>
       <c r="R80" t="n">
-        <v>0.695</v>
+        <v>0.615</v>
       </c>
       <c r="S80" t="n">
-        <v>0.149</v>
+        <v>0.142</v>
       </c>
       <c r="T80" t="n">
-        <v>0.006</v>
+        <v>0.011</v>
       </c>
       <c r="U80" t="n">
-        <v>0.103</v>
+        <v>0.15</v>
       </c>
       <c r="V80" t="n">
-        <v>0.473</v>
+        <v>0.455</v>
       </c>
       <c r="W80" t="n">
-        <v>0.459</v>
+        <v>0.572</v>
       </c>
       <c r="X80" t="n">
-        <v>0.024</v>
+        <v>0.282</v>
       </c>
       <c r="Y80" t="n">
-        <v>0.018</v>
+        <v>0.22</v>
       </c>
       <c r="Z80" t="n">
-        <v>6.465</v>
+        <v>8.191000000000001</v>
       </c>
       <c r="AA80" t="n">
-        <v>8.406000000000001</v>
+        <v>10.682</v>
       </c>
       <c r="AB80" t="n">
-        <v>0.099</v>
+        <v>0.139</v>
       </c>
       <c r="AC80" t="n">
-        <v>0.652</v>
+        <v>0.631</v>
       </c>
       <c r="AD80" t="n">
-        <v>0.018</v>
+        <v>0.202</v>
       </c>
     </row>
     <row r="81">
@@ -9111,16 +9111,16 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>665487</v>
+        <v>666023</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Fernando Tatis Jr.</t>
+          <t>Freddy Fermin</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Tatis Jr.</t>
+          <t>Fermin</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -9144,64 +9144,64 @@
         </is>
       </c>
       <c r="K81" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="L81" t="n">
-        <v>4.355</v>
+        <v>3.363</v>
       </c>
       <c r="M81" t="n">
-        <v>3.788</v>
+        <v>3.035</v>
       </c>
       <c r="N81" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.716</v>
       </c>
       <c r="O81" t="n">
-        <v>1.578</v>
+        <v>1.051</v>
       </c>
       <c r="P81" t="n">
-        <v>0.958</v>
+        <v>0.616</v>
       </c>
       <c r="Q81" t="n">
-        <v>0.476</v>
+        <v>0.247</v>
       </c>
       <c r="R81" t="n">
-        <v>0.623</v>
+        <v>0.518</v>
       </c>
       <c r="S81" t="n">
-        <v>0.155</v>
+        <v>0.129</v>
       </c>
       <c r="T81" t="n">
-        <v>0.008999999999999999</v>
+        <v>0</v>
       </c>
       <c r="U81" t="n">
-        <v>0.154</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="V81" t="n">
-        <v>0.494</v>
+        <v>0.312</v>
       </c>
       <c r="W81" t="n">
-        <v>0.606</v>
+        <v>0.368</v>
       </c>
       <c r="X81" t="n">
-        <v>0.293</v>
+        <v>0.021</v>
       </c>
       <c r="Y81" t="n">
-        <v>0.222</v>
+        <v>0.016</v>
       </c>
       <c r="Z81" t="n">
-        <v>8.525</v>
+        <v>4.822</v>
       </c>
       <c r="AA81" t="n">
-        <v>11.164</v>
+        <v>6.262</v>
       </c>
       <c r="AB81" t="n">
-        <v>0.143</v>
+        <v>0.066</v>
       </c>
       <c r="AC81" t="n">
-        <v>0.654</v>
+        <v>0.534</v>
       </c>
       <c r="AD81" t="n">
-        <v>0.201</v>
+        <v>0.016</v>
       </c>
     </row>
     <row r="82">
@@ -9252,61 +9252,61 @@
         </is>
       </c>
       <c r="K82" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L82" t="n">
-        <v>4.261</v>
+        <v>4.198</v>
       </c>
       <c r="M82" t="n">
-        <v>3.962</v>
+        <v>3.926</v>
       </c>
       <c r="N82" t="n">
-        <v>0.729</v>
+        <v>0.751</v>
       </c>
       <c r="O82" t="n">
-        <v>1.33</v>
+        <v>1.343</v>
       </c>
       <c r="P82" t="n">
-        <v>1.303</v>
+        <v>1.262</v>
       </c>
       <c r="Q82" t="n">
-        <v>0.202</v>
+        <v>0.188</v>
       </c>
       <c r="R82" t="n">
-        <v>0.456</v>
+        <v>0.469</v>
       </c>
       <c r="S82" t="n">
-        <v>0.098</v>
+        <v>0.111</v>
       </c>
       <c r="T82" t="n">
-        <v>0.023</v>
+        <v>0.03</v>
       </c>
       <c r="U82" t="n">
-        <v>0.152</v>
+        <v>0.14</v>
       </c>
       <c r="V82" t="n">
-        <v>0.391</v>
+        <v>0.418</v>
       </c>
       <c r="W82" t="n">
-        <v>0.365</v>
+        <v>0.345</v>
       </c>
       <c r="X82" t="n">
-        <v>0.096</v>
+        <v>0.103</v>
       </c>
       <c r="Y82" t="n">
         <v>0.083</v>
       </c>
       <c r="Z82" t="n">
-        <v>5.892</v>
+        <v>5.922</v>
       </c>
       <c r="AA82" t="n">
-        <v>7.625</v>
+        <v>7.655</v>
       </c>
       <c r="AB82" t="n">
-        <v>0.142</v>
+        <v>0.133</v>
       </c>
       <c r="AC82" t="n">
-        <v>0.521</v>
+        <v>0.55</v>
       </c>
       <c r="AD82" t="n">
         <v>0.08</v>
@@ -9363,61 +9363,61 @@
         <v>1</v>
       </c>
       <c r="L83" t="n">
-        <v>4.222</v>
+        <v>4.258</v>
       </c>
       <c r="M83" t="n">
-        <v>3.62</v>
+        <v>3.637</v>
       </c>
       <c r="N83" t="n">
-        <v>0.6909999999999999</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="O83" t="n">
-        <v>1.145</v>
+        <v>1.127</v>
       </c>
       <c r="P83" t="n">
-        <v>1.453</v>
+        <v>1.462</v>
       </c>
       <c r="Q83" t="n">
-        <v>0.513</v>
+        <v>0.541</v>
       </c>
       <c r="R83" t="n">
-        <v>0.47</v>
+        <v>0.466</v>
       </c>
       <c r="S83" t="n">
-        <v>0.102</v>
+        <v>0.098</v>
       </c>
       <c r="T83" t="n">
         <v>0.006</v>
       </c>
       <c r="U83" t="n">
-        <v>0.114</v>
+        <v>0.112</v>
       </c>
       <c r="V83" t="n">
-        <v>0.288</v>
+        <v>0.267</v>
       </c>
       <c r="W83" t="n">
-        <v>0.384</v>
+        <v>0.405</v>
       </c>
       <c r="X83" t="n">
-        <v>0.061</v>
+        <v>0.062</v>
       </c>
       <c r="Y83" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Z83" t="n">
+        <v>5.728</v>
+      </c>
+      <c r="AA83" t="n">
+        <v>7.533</v>
+      </c>
+      <c r="AB83" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="AC83" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AD83" t="n">
         <v>0.049</v>
-      </c>
-      <c r="Z83" t="n">
-        <v>5.718</v>
-      </c>
-      <c r="AA83" t="n">
-        <v>7.508</v>
-      </c>
-      <c r="AB83" t="n">
-        <v>0.109</v>
-      </c>
-      <c r="AC83" t="n">
-        <v>0.509</v>
-      </c>
-      <c r="AD83" t="n">
-        <v>0.048</v>
       </c>
     </row>
     <row r="84">
@@ -9435,21 +9435,21 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>669134</v>
+        <v>669369</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Luis Campusano</t>
+          <t>Bryce Johnson</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Campusano</t>
+          <t>Johnson</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -9468,64 +9468,64 @@
         </is>
       </c>
       <c r="K84" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L84" t="n">
-        <v>3.422</v>
+        <v>3.652</v>
       </c>
       <c r="M84" t="n">
-        <v>3.098</v>
+        <v>3.353</v>
       </c>
       <c r="N84" t="n">
-        <v>0.724</v>
+        <v>0.805</v>
       </c>
       <c r="O84" t="n">
-        <v>1.095</v>
+        <v>1.225</v>
       </c>
       <c r="P84" t="n">
-        <v>0.643</v>
+        <v>0.76</v>
       </c>
       <c r="Q84" t="n">
-        <v>0.238</v>
+        <v>0.215</v>
       </c>
       <c r="R84" t="n">
-        <v>0.519</v>
+        <v>0.575</v>
       </c>
       <c r="S84" t="n">
-        <v>0.123</v>
+        <v>0.136</v>
       </c>
       <c r="T84" t="n">
         <v>0</v>
       </c>
       <c r="U84" t="n">
-        <v>0.082</v>
+        <v>0.095</v>
       </c>
       <c r="V84" t="n">
-        <v>0.385</v>
+        <v>0.388</v>
       </c>
       <c r="W84" t="n">
-        <v>0.37</v>
+        <v>0.412</v>
       </c>
       <c r="X84" t="n">
-        <v>0.006</v>
+        <v>0.179</v>
       </c>
       <c r="Y84" t="n">
-        <v>0.004</v>
+        <v>0.142</v>
       </c>
       <c r="Z84" t="n">
-        <v>5.003</v>
+        <v>6.087</v>
       </c>
       <c r="AA84" t="n">
-        <v>6.555</v>
+        <v>7.845</v>
       </c>
       <c r="AB84" t="n">
-        <v>0.079</v>
+        <v>0.09</v>
       </c>
       <c r="AC84" t="n">
-        <v>0.543</v>
+        <v>0.576</v>
       </c>
       <c r="AD84" t="n">
-        <v>0.004</v>
+        <v>0.135</v>
       </c>
     </row>
     <row r="85">
@@ -9543,16 +9543,16 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>678662</v>
+        <v>671289</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Ezequiel Tovar</t>
+          <t>Tyler Freeman</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Tovar</t>
+          <t>Freeman</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -9576,64 +9576,64 @@
         </is>
       </c>
       <c r="K85" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L85" t="n">
-        <v>4.165</v>
+        <v>4.445</v>
       </c>
       <c r="M85" t="n">
-        <v>3.845</v>
+        <v>4.004</v>
       </c>
       <c r="N85" t="n">
-        <v>0.751</v>
+        <v>0.923</v>
       </c>
       <c r="O85" t="n">
-        <v>1.314</v>
+        <v>1.332</v>
       </c>
       <c r="P85" t="n">
-        <v>1.303</v>
+        <v>0.6879999999999999</v>
       </c>
       <c r="Q85" t="n">
-        <v>0.228</v>
+        <v>0.337</v>
       </c>
       <c r="R85" t="n">
-        <v>0.477</v>
+        <v>0.678</v>
       </c>
       <c r="S85" t="n">
-        <v>0.121</v>
+        <v>0.16</v>
       </c>
       <c r="T85" t="n">
-        <v>0.014</v>
+        <v>0.006</v>
       </c>
       <c r="U85" t="n">
-        <v>0.138</v>
+        <v>0.079</v>
       </c>
       <c r="V85" t="n">
-        <v>0.372</v>
+        <v>0.326</v>
       </c>
       <c r="W85" t="n">
-        <v>0.336</v>
+        <v>0.39</v>
       </c>
       <c r="X85" t="n">
-        <v>0.061</v>
+        <v>0.188</v>
       </c>
       <c r="Y85" t="n">
-        <v>0.052</v>
+        <v>0.155</v>
       </c>
       <c r="Z85" t="n">
-        <v>5.664</v>
+        <v>6.552</v>
       </c>
       <c r="AA85" t="n">
-        <v>7.317</v>
+        <v>8.324</v>
       </c>
       <c r="AB85" t="n">
-        <v>0.132</v>
+        <v>0.076</v>
       </c>
       <c r="AC85" t="n">
-        <v>0.551</v>
+        <v>0.627</v>
       </c>
       <c r="AD85" t="n">
-        <v>0.051</v>
+        <v>0.145</v>
       </c>
     </row>
     <row r="86">
@@ -9651,21 +9651,21 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>681198</v>
+        <v>678662</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>TJ Rumfield</t>
+          <t>Ezequiel Tovar</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Rumfield</t>
+          <t>Tovar</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -9684,64 +9684,64 @@
         </is>
       </c>
       <c r="K86" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L86" t="n">
-        <v>4.101</v>
+        <v>4.023</v>
       </c>
       <c r="M86" t="n">
-        <v>3.678</v>
+        <v>3.73</v>
       </c>
       <c r="N86" t="n">
-        <v>0.612</v>
+        <v>0.725</v>
       </c>
       <c r="O86" t="n">
-        <v>0.958</v>
+        <v>1.301</v>
       </c>
       <c r="P86" t="n">
-        <v>1.214</v>
+        <v>1.286</v>
       </c>
       <c r="Q86" t="n">
-        <v>0.337</v>
+        <v>0.211</v>
       </c>
       <c r="R86" t="n">
-        <v>0.416</v>
+        <v>0.447</v>
       </c>
       <c r="S86" t="n">
-        <v>0.119</v>
+        <v>0.123</v>
       </c>
       <c r="T86" t="n">
-        <v>0.006</v>
+        <v>0.011</v>
       </c>
       <c r="U86" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.144</v>
       </c>
       <c r="V86" t="n">
-        <v>0.267</v>
+        <v>0.385</v>
       </c>
       <c r="W86" t="n">
-        <v>0.279</v>
+        <v>0.344</v>
       </c>
       <c r="X86" t="n">
-        <v>0.041</v>
+        <v>0.05</v>
       </c>
       <c r="Y86" t="n">
-        <v>0.031</v>
+        <v>0.043</v>
       </c>
       <c r="Z86" t="n">
-        <v>4.527</v>
+        <v>5.578</v>
       </c>
       <c r="AA86" t="n">
-        <v>5.898</v>
+        <v>7.243</v>
       </c>
       <c r="AB86" t="n">
-        <v>0.068</v>
+        <v>0.14</v>
       </c>
       <c r="AC86" t="n">
-        <v>0.471</v>
+        <v>0.545</v>
       </c>
       <c r="AD86" t="n">
-        <v>0.03</v>
+        <v>0.042</v>
       </c>
     </row>
     <row r="87">
@@ -9759,21 +9759,21 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>686668</v>
+        <v>681198</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Brenton Doyle</t>
+          <t>TJ Rumfield</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Doyle</t>
+          <t>Rumfield</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -9792,64 +9792,64 @@
         </is>
       </c>
       <c r="K87" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="L87" t="n">
-        <v>3.704</v>
+        <v>3.993</v>
       </c>
       <c r="M87" t="n">
-        <v>3.371</v>
+        <v>3.584</v>
       </c>
       <c r="N87" t="n">
-        <v>0.61</v>
+        <v>0.599</v>
       </c>
       <c r="O87" t="n">
-        <v>0.964</v>
+        <v>0.919</v>
       </c>
       <c r="P87" t="n">
-        <v>1.231</v>
+        <v>1.162</v>
       </c>
       <c r="Q87" t="n">
-        <v>0.25</v>
+        <v>0.321</v>
       </c>
       <c r="R87" t="n">
         <v>0.422</v>
       </c>
       <c r="S87" t="n">
-        <v>0.1</v>
+        <v>0.103</v>
       </c>
       <c r="T87" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.005</v>
       </c>
       <c r="U87" t="n">
-        <v>0.079</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="V87" t="n">
-        <v>0.262</v>
+        <v>0.255</v>
       </c>
       <c r="W87" t="n">
-        <v>0.277</v>
+        <v>0.281</v>
       </c>
       <c r="X87" t="n">
-        <v>0.164</v>
+        <v>0.04</v>
       </c>
       <c r="Y87" t="n">
-        <v>0.138</v>
+        <v>0.033</v>
       </c>
       <c r="Z87" t="n">
-        <v>4.896</v>
+        <v>4.386</v>
       </c>
       <c r="AA87" t="n">
-        <v>6.277</v>
+        <v>5.705</v>
       </c>
       <c r="AB87" t="n">
-        <v>0.077</v>
+        <v>0.067</v>
       </c>
       <c r="AC87" t="n">
-        <v>0.466</v>
+        <v>0.464</v>
       </c>
       <c r="AD87" t="n">
-        <v>0.13</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="88">
@@ -9867,21 +9867,21 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>687859</v>
+        <v>686668</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Troy Johnston</t>
+          <t>Brenton Doyle</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Johnston</t>
+          <t>Doyle</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -9900,64 +9900,64 @@
         </is>
       </c>
       <c r="K88" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L88" t="n">
-        <v>3.689</v>
+        <v>3.856</v>
       </c>
       <c r="M88" t="n">
-        <v>3.359</v>
+        <v>3.517</v>
       </c>
       <c r="N88" t="n">
-        <v>0.575</v>
+        <v>0.634</v>
       </c>
       <c r="O88" t="n">
-        <v>0.931</v>
+        <v>0.994</v>
       </c>
       <c r="P88" t="n">
-        <v>1.101</v>
+        <v>1.252</v>
       </c>
       <c r="Q88" t="n">
-        <v>0.249</v>
+        <v>0.255</v>
       </c>
       <c r="R88" t="n">
-        <v>0.391</v>
+        <v>0.448</v>
       </c>
       <c r="S88" t="n">
-        <v>0.096</v>
+        <v>0.091</v>
       </c>
       <c r="T88" t="n">
-        <v>0.006</v>
+        <v>0.013</v>
       </c>
       <c r="U88" t="n">
-        <v>0.083</v>
+        <v>0.081</v>
       </c>
       <c r="V88" t="n">
-        <v>0.247</v>
+        <v>0.269</v>
       </c>
       <c r="W88" t="n">
-        <v>0.258</v>
+        <v>0.276</v>
       </c>
       <c r="X88" t="n">
-        <v>0.079</v>
+        <v>0.183</v>
       </c>
       <c r="Y88" t="n">
-        <v>0.06</v>
+        <v>0.146</v>
       </c>
       <c r="Z88" t="n">
-        <v>4.332</v>
+        <v>5.044</v>
       </c>
       <c r="AA88" t="n">
-        <v>5.588</v>
+        <v>6.445</v>
       </c>
       <c r="AB88" t="n">
-        <v>0.08</v>
+        <v>0.077</v>
       </c>
       <c r="AC88" t="n">
-        <v>0.459</v>
+        <v>0.48</v>
       </c>
       <c r="AD88" t="n">
-        <v>0.058</v>
+        <v>0.138</v>
       </c>
     </row>
     <row r="89">
@@ -10011,61 +10011,61 @@
         <v>9</v>
       </c>
       <c r="L89" t="n">
-        <v>3.614</v>
+        <v>3.627</v>
       </c>
       <c r="M89" t="n">
-        <v>3.181</v>
+        <v>3.18</v>
       </c>
       <c r="N89" t="n">
-        <v>0.575</v>
+        <v>0.592</v>
       </c>
       <c r="O89" t="n">
-        <v>0.866</v>
+        <v>0.89</v>
       </c>
       <c r="P89" t="n">
-        <v>1.213</v>
+        <v>1.223</v>
       </c>
       <c r="Q89" t="n">
-        <v>0.367</v>
+        <v>0.378</v>
       </c>
       <c r="R89" t="n">
-        <v>0.414</v>
+        <v>0.431</v>
       </c>
       <c r="S89" t="n">
-        <v>0.097</v>
+        <v>0.093</v>
       </c>
       <c r="T89" t="n">
         <v>0</v>
       </c>
       <c r="U89" t="n">
-        <v>0.064</v>
+        <v>0.068</v>
       </c>
       <c r="V89" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="W89" t="n">
-        <v>0.28</v>
+        <v>0.292</v>
       </c>
       <c r="X89" t="n">
-        <v>0.045</v>
+        <v>0.043</v>
       </c>
       <c r="Y89" t="n">
-        <v>0.034</v>
+        <v>0.037</v>
       </c>
       <c r="Z89" t="n">
-        <v>4.318</v>
+        <v>4.426</v>
       </c>
       <c r="AA89" t="n">
-        <v>5.642</v>
+        <v>5.766</v>
       </c>
       <c r="AB89" t="n">
-        <v>0.063</v>
+        <v>0.067</v>
       </c>
       <c r="AC89" t="n">
-        <v>0.458</v>
+        <v>0.463</v>
       </c>
       <c r="AD89" t="n">
-        <v>0.033</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="90">
@@ -10116,64 +10116,64 @@
         </is>
       </c>
       <c r="K90" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L90" t="n">
-        <v>4.24</v>
+        <v>4.191</v>
       </c>
       <c r="M90" t="n">
-        <v>3.784</v>
+        <v>3.756</v>
       </c>
       <c r="N90" t="n">
-        <v>0.675</v>
+        <v>0.659</v>
       </c>
       <c r="O90" t="n">
-        <v>1.275</v>
+        <v>1.24</v>
       </c>
       <c r="P90" t="n">
-        <v>1.414</v>
+        <v>1.4</v>
       </c>
       <c r="Q90" t="n">
-        <v>0.355</v>
+        <v>0.348</v>
       </c>
       <c r="R90" t="n">
-        <v>0.396</v>
+        <v>0.39</v>
       </c>
       <c r="S90" t="n">
-        <v>0.111</v>
+        <v>0.102</v>
       </c>
       <c r="T90" t="n">
-        <v>0.015</v>
+        <v>0.019</v>
       </c>
       <c r="U90" t="n">
-        <v>0.153</v>
+        <v>0.147</v>
       </c>
       <c r="V90" t="n">
-        <v>0.367</v>
+        <v>0.406</v>
       </c>
       <c r="W90" t="n">
-        <v>0.352</v>
+        <v>0.35</v>
       </c>
       <c r="X90" t="n">
-        <v>0.047</v>
+        <v>0.044</v>
       </c>
       <c r="Y90" t="n">
-        <v>0.036</v>
+        <v>0.035</v>
       </c>
       <c r="Z90" t="n">
-        <v>5.72</v>
+        <v>5.687</v>
       </c>
       <c r="AA90" t="n">
-        <v>7.516</v>
+        <v>7.515</v>
       </c>
       <c r="AB90" t="n">
-        <v>0.141</v>
+        <v>0.138</v>
       </c>
       <c r="AC90" t="n">
-        <v>0.51</v>
+        <v>0.501</v>
       </c>
       <c r="AD90" t="n">
-        <v>0.035</v>
+        <v>0.034</v>
       </c>
     </row>
     <row r="91">
@@ -10227,61 +10227,61 @@
         <v>3</v>
       </c>
       <c r="L91" t="n">
-        <v>4.345</v>
+        <v>4.346</v>
       </c>
       <c r="M91" t="n">
-        <v>3.901</v>
+        <v>3.892</v>
       </c>
       <c r="N91" t="n">
-        <v>1.01</v>
+        <v>1.003</v>
       </c>
       <c r="O91" t="n">
-        <v>1.7</v>
+        <v>1.638</v>
       </c>
       <c r="P91" t="n">
-        <v>0.845</v>
+        <v>0.831</v>
       </c>
       <c r="Q91" t="n">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="R91" t="n">
-        <v>0.661</v>
+        <v>0.674</v>
       </c>
       <c r="S91" t="n">
         <v>0.161</v>
       </c>
       <c r="T91" t="n">
-        <v>0.037</v>
+        <v>0.03</v>
       </c>
       <c r="U91" t="n">
-        <v>0.152</v>
+        <v>0.138</v>
       </c>
       <c r="V91" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.53</v>
       </c>
       <c r="W91" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.524</v>
       </c>
       <c r="X91" t="n">
-        <v>0.123</v>
+        <v>0.118</v>
       </c>
       <c r="Y91" t="n">
-        <v>0.095</v>
+        <v>0.098</v>
       </c>
       <c r="Z91" t="n">
-        <v>7.995</v>
+        <v>7.746</v>
       </c>
       <c r="AA91" t="n">
-        <v>10.444</v>
+        <v>10.086</v>
       </c>
       <c r="AB91" t="n">
-        <v>0.143</v>
+        <v>0.13</v>
       </c>
       <c r="AC91" t="n">
-        <v>0.666</v>
+        <v>0.674</v>
       </c>
       <c r="AD91" t="n">
-        <v>0.091</v>
+        <v>0.094</v>
       </c>
     </row>
     <row r="92">
@@ -16167,61 +16167,61 @@
         <v>4</v>
       </c>
       <c r="L146" t="n">
-        <v>4.058</v>
+        <v>4.059</v>
       </c>
       <c r="M146" t="n">
-        <v>3.611</v>
+        <v>3.597</v>
       </c>
       <c r="N146" t="n">
-        <v>0.784</v>
+        <v>0.768</v>
       </c>
       <c r="O146" t="n">
-        <v>1.399</v>
+        <v>1.342</v>
       </c>
       <c r="P146" t="n">
-        <v>0.93</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="Q146" t="n">
-        <v>0.361</v>
+        <v>0.375</v>
       </c>
       <c r="R146" t="n">
-        <v>0.467</v>
+        <v>0.47</v>
       </c>
       <c r="S146" t="n">
-        <v>0.163</v>
+        <v>0.157</v>
       </c>
       <c r="T146" t="n">
         <v>0.008</v>
       </c>
       <c r="U146" t="n">
-        <v>0.145</v>
+        <v>0.134</v>
       </c>
       <c r="V146" t="n">
-        <v>0.466</v>
+        <v>0.413</v>
       </c>
       <c r="W146" t="n">
-        <v>0.434</v>
+        <v>0.401</v>
       </c>
       <c r="X146" t="n">
-        <v>0.052</v>
+        <v>0.055</v>
       </c>
       <c r="Y146" t="n">
-        <v>0.041</v>
+        <v>0.045</v>
       </c>
       <c r="Z146" t="n">
-        <v>6.465</v>
+        <v>6.196</v>
       </c>
       <c r="AA146" t="n">
-        <v>8.550000000000001</v>
+        <v>8.148</v>
       </c>
       <c r="AB146" t="n">
-        <v>0.136</v>
+        <v>0.129</v>
       </c>
       <c r="AC146" t="n">
-        <v>0.571</v>
+        <v>0.572</v>
       </c>
       <c r="AD146" t="n">
-        <v>0.04</v>
+        <v>0.045</v>
       </c>
     </row>
     <row r="147">
@@ -16275,61 +16275,61 @@
         <v>5</v>
       </c>
       <c r="L147" t="n">
-        <v>4.062</v>
+        <v>4.023</v>
       </c>
       <c r="M147" t="n">
-        <v>3.525</v>
+        <v>3.49</v>
       </c>
       <c r="N147" t="n">
-        <v>0.6820000000000001</v>
+        <v>0.7</v>
       </c>
       <c r="O147" t="n">
-        <v>1.279</v>
+        <v>1.323</v>
       </c>
       <c r="P147" t="n">
-        <v>1.197</v>
+        <v>1.185</v>
       </c>
       <c r="Q147" t="n">
-        <v>0.455</v>
+        <v>0.454</v>
       </c>
       <c r="R147" t="n">
-        <v>0.397</v>
+        <v>0.404</v>
       </c>
       <c r="S147" t="n">
-        <v>0.126</v>
+        <v>0.129</v>
       </c>
       <c r="T147" t="n">
         <v>0.006</v>
       </c>
       <c r="U147" t="n">
-        <v>0.153</v>
+        <v>0.16</v>
       </c>
       <c r="V147" t="n">
-        <v>0.443</v>
+        <v>0.43</v>
       </c>
       <c r="W147" t="n">
-        <v>0.416</v>
+        <v>0.391</v>
       </c>
       <c r="X147" t="n">
-        <v>0.037</v>
+        <v>0.034</v>
       </c>
       <c r="Y147" t="n">
-        <v>0.029</v>
+        <v>0.025</v>
       </c>
       <c r="Z147" t="n">
-        <v>6.171</v>
+        <v>6.187</v>
       </c>
       <c r="AA147" t="n">
-        <v>8.257</v>
+        <v>8.236000000000001</v>
       </c>
       <c r="AB147" t="n">
-        <v>0.143</v>
+        <v>0.15</v>
       </c>
       <c r="AC147" t="n">
-        <v>0.511</v>
+        <v>0.528</v>
       </c>
       <c r="AD147" t="n">
-        <v>0.029</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="148">
@@ -16383,61 +16383,61 @@
         <v>5</v>
       </c>
       <c r="L148" t="n">
-        <v>4.243</v>
+        <v>4.237</v>
       </c>
       <c r="M148" t="n">
-        <v>3.584</v>
+        <v>3.605</v>
       </c>
       <c r="N148" t="n">
-        <v>0.753</v>
+        <v>0.758</v>
       </c>
       <c r="O148" t="n">
-        <v>1.314</v>
+        <v>1.328</v>
       </c>
       <c r="P148" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.967</v>
       </c>
       <c r="Q148" t="n">
-        <v>0.57</v>
+        <v>0.545</v>
       </c>
       <c r="R148" t="n">
-        <v>0.46</v>
+        <v>0.461</v>
       </c>
       <c r="S148" t="n">
-        <v>0.154</v>
+        <v>0.155</v>
       </c>
       <c r="T148" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="U148" t="n">
-        <v>0.128</v>
+        <v>0.131</v>
       </c>
       <c r="V148" t="n">
-        <v>0.472</v>
+        <v>0.489</v>
       </c>
       <c r="W148" t="n">
-        <v>0.467</v>
+        <v>0.475</v>
       </c>
       <c r="X148" t="n">
-        <v>0.046</v>
+        <v>0.052</v>
       </c>
       <c r="Y148" t="n">
-        <v>0.034</v>
+        <v>0.041</v>
       </c>
       <c r="Z148" t="n">
-        <v>6.708</v>
+        <v>6.78</v>
       </c>
       <c r="AA148" t="n">
-        <v>9</v>
+        <v>9.097</v>
       </c>
       <c r="AB148" t="n">
-        <v>0.121</v>
+        <v>0.123</v>
       </c>
       <c r="AC148" t="n">
         <v>0.55</v>
       </c>
       <c r="AD148" t="n">
-        <v>0.033</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="149">
@@ -16455,97 +16455,97 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>606192</v>
+        <v>607043</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Teoscar Hernandez</t>
+          <t>Brandon Nimmo</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>Hernandez</t>
+          <t>Nimmo</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
+          <t>TEX</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
           <t>LAD</t>
         </is>
       </c>
-      <c r="J149" t="inlineStr">
-        <is>
-          <t>TEX</t>
-        </is>
-      </c>
       <c r="K149" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L149" t="n">
-        <v>3.881</v>
+        <v>4.854</v>
       </c>
       <c r="M149" t="n">
-        <v>3.523</v>
+        <v>4.145</v>
       </c>
       <c r="N149" t="n">
-        <v>0.771</v>
+        <v>0.966</v>
       </c>
       <c r="O149" t="n">
-        <v>1.303</v>
+        <v>1.659</v>
       </c>
       <c r="P149" t="n">
-        <v>1.103</v>
+        <v>0.991</v>
       </c>
       <c r="Q149" t="n">
-        <v>0.272</v>
+        <v>0.599</v>
       </c>
       <c r="R149" t="n">
-        <v>0.487</v>
+        <v>0.611</v>
       </c>
       <c r="S149" t="n">
-        <v>0.155</v>
+        <v>0.174</v>
       </c>
       <c r="T149" t="n">
-        <v>0.01</v>
+        <v>0.023</v>
       </c>
       <c r="U149" t="n">
-        <v>0.119</v>
+        <v>0.158</v>
       </c>
       <c r="V149" t="n">
-        <v>0.409</v>
+        <v>0.481</v>
       </c>
       <c r="W149" t="n">
-        <v>0.343</v>
+        <v>0.638</v>
       </c>
       <c r="X149" t="n">
-        <v>0.099</v>
+        <v>0.102</v>
       </c>
       <c r="Y149" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="Z149" t="n">
+        <v>8.324999999999999</v>
+      </c>
+      <c r="AA149" t="n">
+        <v>11.008</v>
+      </c>
+      <c r="AB149" t="n">
+        <v>0.148</v>
+      </c>
+      <c r="AC149" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="AD149" t="n">
         <v>0.082</v>
-      </c>
-      <c r="Z149" t="n">
-        <v>5.965</v>
-      </c>
-      <c r="AA149" t="n">
-        <v>7.747</v>
-      </c>
-      <c r="AB149" t="n">
-        <v>0.113</v>
-      </c>
-      <c r="AC149" t="n">
-        <v>0.556</v>
-      </c>
-      <c r="AD149" t="n">
-        <v>0.08</v>
       </c>
     </row>
     <row r="150">
@@ -16563,16 +16563,16 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>607043</v>
+        <v>608369</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Brandon Nimmo</t>
+          <t>Corey Seager</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>Nimmo</t>
+          <t>Seager</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -16596,64 +16596,64 @@
         </is>
       </c>
       <c r="K150" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L150" t="n">
-        <v>4.862</v>
+        <v>4.644</v>
       </c>
       <c r="M150" t="n">
-        <v>4.174</v>
+        <v>3.864</v>
       </c>
       <c r="N150" t="n">
-        <v>0.952</v>
+        <v>0.979</v>
       </c>
       <c r="O150" t="n">
-        <v>1.641</v>
+        <v>1.784</v>
       </c>
       <c r="P150" t="n">
-        <v>0.973</v>
+        <v>0.948</v>
       </c>
       <c r="Q150" t="n">
-        <v>0.581</v>
+        <v>0.678</v>
       </c>
       <c r="R150" t="n">
-        <v>0.591</v>
+        <v>0.572</v>
       </c>
       <c r="S150" t="n">
-        <v>0.181</v>
+        <v>0.204</v>
       </c>
       <c r="T150" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="U150" t="n">
+        <v>0.194</v>
+      </c>
+      <c r="V150" t="n">
+        <v>0.649</v>
+      </c>
+      <c r="W150" t="n">
+        <v>0.588</v>
+      </c>
+      <c r="X150" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="Y150" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="Z150" t="n">
+        <v>8.728999999999999</v>
+      </c>
+      <c r="AA150" t="n">
+        <v>11.718</v>
+      </c>
+      <c r="AB150" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="AC150" t="n">
+        <v>0.652</v>
+      </c>
+      <c r="AD150" t="n">
         <v>0.029</v>
-      </c>
-      <c r="U150" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="V150" t="n">
-        <v>0.485</v>
-      </c>
-      <c r="W150" t="n">
-        <v>0.645</v>
-      </c>
-      <c r="X150" t="n">
-        <v>0.101</v>
-      </c>
-      <c r="Y150" t="n">
-        <v>0.082</v>
-      </c>
-      <c r="Z150" t="n">
-        <v>8.244999999999999</v>
-      </c>
-      <c r="AA150" t="n">
-        <v>10.919</v>
-      </c>
-      <c r="AB150" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="AC150" t="n">
-        <v>0.638</v>
-      </c>
-      <c r="AD150" t="n">
-        <v>0.081</v>
       </c>
     </row>
     <row r="151">
@@ -16671,21 +16671,21 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>608369</v>
+        <v>643376</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Corey Seager</t>
+          <t>Danny Jansen</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>Seager</t>
+          <t>Jansen</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -16704,64 +16704,64 @@
         </is>
       </c>
       <c r="K151" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L151" t="n">
-        <v>4.656</v>
+        <v>4.309</v>
       </c>
       <c r="M151" t="n">
-        <v>3.896</v>
+        <v>3.635</v>
       </c>
       <c r="N151" t="n">
-        <v>0.981</v>
+        <v>0.728</v>
       </c>
       <c r="O151" t="n">
-        <v>1.777</v>
+        <v>1.281</v>
       </c>
       <c r="P151" t="n">
-        <v>0.959</v>
+        <v>1.142</v>
       </c>
       <c r="Q151" t="n">
-        <v>0.669</v>
+        <v>0.583</v>
       </c>
       <c r="R151" t="n">
-        <v>0.576</v>
+        <v>0.439</v>
       </c>
       <c r="S151" t="n">
-        <v>0.204</v>
+        <v>0.156</v>
       </c>
       <c r="T151" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.002</v>
       </c>
       <c r="U151" t="n">
-        <v>0.191</v>
+        <v>0.131</v>
       </c>
       <c r="V151" t="n">
-        <v>0.648</v>
+        <v>0.435</v>
       </c>
       <c r="W151" t="n">
-        <v>0.577</v>
+        <v>0.458</v>
       </c>
       <c r="X151" t="n">
-        <v>0.039</v>
+        <v>0.021</v>
       </c>
       <c r="Y151" t="n">
-        <v>0.03</v>
+        <v>0.017</v>
       </c>
       <c r="Z151" t="n">
-        <v>8.673</v>
+        <v>6.461</v>
       </c>
       <c r="AA151" t="n">
-        <v>11.633</v>
+        <v>8.683999999999999</v>
       </c>
       <c r="AB151" t="n">
-        <v>0.177</v>
+        <v>0.122</v>
       </c>
       <c r="AC151" t="n">
-        <v>0.658</v>
+        <v>0.54</v>
       </c>
       <c r="AD151" t="n">
-        <v>0.029</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="152">
@@ -16779,97 +16779,97 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>643376</v>
+        <v>660271</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Danny Jansen</t>
+          <t>Shohei Ohtani</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>Jansen</t>
+          <t>Ohtani</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
         <is>
+          <t>LAD</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
           <t>TEX</t>
         </is>
       </c>
-      <c r="J152" t="inlineStr">
-        <is>
-          <t>LAD</t>
-        </is>
-      </c>
       <c r="K152" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L152" t="n">
-        <v>4.235</v>
+        <v>4.487</v>
       </c>
       <c r="M152" t="n">
-        <v>3.574</v>
+        <v>3.91</v>
       </c>
       <c r="N152" t="n">
-        <v>0.74</v>
+        <v>0.803</v>
       </c>
       <c r="O152" t="n">
-        <v>1.277</v>
+        <v>1.742</v>
       </c>
       <c r="P152" t="n">
-        <v>1.112</v>
+        <v>1.514</v>
       </c>
       <c r="Q152" t="n">
-        <v>0.576</v>
+        <v>0.484</v>
       </c>
       <c r="R152" t="n">
-        <v>0.453</v>
+        <v>0.403</v>
       </c>
       <c r="S152" t="n">
-        <v>0.16</v>
+        <v>0.113</v>
       </c>
       <c r="T152" t="n">
-        <v>0.002</v>
+        <v>0.034</v>
       </c>
       <c r="U152" t="n">
-        <v>0.125</v>
+        <v>0.253</v>
       </c>
       <c r="V152" t="n">
-        <v>0.463</v>
+        <v>0.511</v>
       </c>
       <c r="W152" t="n">
-        <v>0.475</v>
+        <v>0.593</v>
       </c>
       <c r="X152" t="n">
-        <v>0.02</v>
+        <v>0.226</v>
       </c>
       <c r="Y152" t="n">
-        <v>0.016</v>
+        <v>0.19</v>
       </c>
       <c r="Z152" t="n">
-        <v>6.528</v>
+        <v>8.702999999999999</v>
       </c>
       <c r="AA152" t="n">
-        <v>8.795</v>
+        <v>11.508</v>
       </c>
       <c r="AB152" t="n">
-        <v>0.118</v>
+        <v>0.23</v>
       </c>
       <c r="AC152" t="n">
-        <v>0.549</v>
+        <v>0.578</v>
       </c>
       <c r="AD152" t="n">
-        <v>0.016</v>
+        <v>0.177</v>
       </c>
     </row>
     <row r="153">
@@ -16887,16 +16887,16 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>660271</v>
+        <v>663656</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Shohei Ohtani</t>
+          <t>Kyle Tucker</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Ohtani</t>
+          <t>Tucker</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -16920,64 +16920,64 @@
         </is>
       </c>
       <c r="K153" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L153" t="n">
-        <v>4.476</v>
+        <v>4.274</v>
       </c>
       <c r="M153" t="n">
-        <v>3.918</v>
+        <v>3.724</v>
       </c>
       <c r="N153" t="n">
-        <v>0.799</v>
+        <v>0.794</v>
       </c>
       <c r="O153" t="n">
-        <v>1.756</v>
+        <v>1.335</v>
       </c>
       <c r="P153" t="n">
-        <v>1.514</v>
+        <v>0.991</v>
       </c>
       <c r="Q153" t="n">
-        <v>0.48</v>
+        <v>0.459</v>
       </c>
       <c r="R153" t="n">
-        <v>0.391</v>
+        <v>0.531</v>
       </c>
       <c r="S153" t="n">
-        <v>0.118</v>
+        <v>0.115</v>
       </c>
       <c r="T153" t="n">
-        <v>0.029</v>
+        <v>0.018</v>
       </c>
       <c r="U153" t="n">
-        <v>0.26</v>
+        <v>0.13</v>
       </c>
       <c r="V153" t="n">
-        <v>0.497</v>
+        <v>0.371</v>
       </c>
       <c r="W153" t="n">
-        <v>0.594</v>
+        <v>0.45</v>
       </c>
       <c r="X153" t="n">
-        <v>0.207</v>
+        <v>0.232</v>
       </c>
       <c r="Y153" t="n">
-        <v>0.172</v>
+        <v>0.191</v>
       </c>
       <c r="Z153" t="n">
-        <v>8.605</v>
+        <v>7.124</v>
       </c>
       <c r="AA153" t="n">
-        <v>11.383</v>
+        <v>9.262</v>
       </c>
       <c r="AB153" t="n">
-        <v>0.233</v>
+        <v>0.123</v>
       </c>
       <c r="AC153" t="n">
-        <v>0.581</v>
+        <v>0.576</v>
       </c>
       <c r="AD153" t="n">
-        <v>0.16</v>
+        <v>0.174</v>
       </c>
     </row>
     <row r="154">
@@ -16995,97 +16995,97 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>663656</v>
+        <v>669394</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Kyle Tucker</t>
+          <t>Jake Burger</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>Tucker</t>
+          <t>Burger</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
+          <t>TEX</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
           <t>LAD</t>
         </is>
       </c>
-      <c r="J154" t="inlineStr">
-        <is>
-          <t>TEX</t>
-        </is>
-      </c>
       <c r="K154" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L154" t="n">
-        <v>4.277</v>
+        <v>4.459</v>
       </c>
       <c r="M154" t="n">
-        <v>3.731</v>
+        <v>4.098</v>
       </c>
       <c r="N154" t="n">
-        <v>0.805</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="O154" t="n">
-        <v>1.391</v>
+        <v>1.634</v>
       </c>
       <c r="P154" t="n">
-        <v>1.013</v>
+        <v>1.187</v>
       </c>
       <c r="Q154" t="n">
-        <v>0.452</v>
+        <v>0.264</v>
       </c>
       <c r="R154" t="n">
-        <v>0.513</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="S154" t="n">
+        <v>0.214</v>
+      </c>
+      <c r="T154" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="U154" t="n">
+        <v>0.151</v>
+      </c>
+      <c r="V154" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="W154" t="n">
+        <v>0.489</v>
+      </c>
+      <c r="X154" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="Y154" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="Z154" t="n">
+        <v>7.198</v>
+      </c>
+      <c r="AA154" t="n">
+        <v>9.493</v>
+      </c>
+      <c r="AB154" t="n">
         <v>0.139</v>
       </c>
-      <c r="T154" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="U154" t="n">
-        <v>0.139</v>
-      </c>
-      <c r="V154" t="n">
-        <v>0.374</v>
-      </c>
-      <c r="W154" t="n">
-        <v>0.486</v>
-      </c>
-      <c r="X154" t="n">
-        <v>0.214</v>
-      </c>
-      <c r="Y154" t="n">
-        <v>0.176</v>
-      </c>
-      <c r="Z154" t="n">
-        <v>7.245</v>
-      </c>
-      <c r="AA154" t="n">
-        <v>9.449999999999999</v>
-      </c>
-      <c r="AB154" t="n">
-        <v>0.131</v>
-      </c>
       <c r="AC154" t="n">
-        <v>0.58</v>
+        <v>0.633</v>
       </c>
       <c r="AD154" t="n">
-        <v>0.164</v>
+        <v>0.027</v>
       </c>
     </row>
     <row r="155">
@@ -17103,11 +17103,11 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>669257</v>
+        <v>669701</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Will Smith</t>
+          <t>Josh Smith</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -17117,83 +17117,83 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
+          <t>TEX</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
           <t>LAD</t>
         </is>
       </c>
-      <c r="J155" t="inlineStr">
-        <is>
-          <t>TEX</t>
-        </is>
-      </c>
       <c r="K155" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L155" t="n">
-        <v>4.231</v>
+        <v>4.177</v>
       </c>
       <c r="M155" t="n">
-        <v>3.581</v>
+        <v>3.56</v>
       </c>
       <c r="N155" t="n">
-        <v>0.77</v>
+        <v>0.831</v>
       </c>
       <c r="O155" t="n">
-        <v>1.356</v>
+        <v>1.336</v>
       </c>
       <c r="P155" t="n">
-        <v>1.112</v>
+        <v>0.737</v>
       </c>
       <c r="Q155" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.532</v>
       </c>
       <c r="R155" t="n">
-        <v>0.481</v>
+        <v>0.528</v>
       </c>
       <c r="S155" t="n">
-        <v>0.134</v>
+        <v>0.195</v>
       </c>
       <c r="T155" t="n">
-        <v>0.012</v>
+        <v>0.013</v>
       </c>
       <c r="U155" t="n">
-        <v>0.143</v>
+        <v>0.094</v>
       </c>
       <c r="V155" t="n">
-        <v>0.43</v>
+        <v>0.425</v>
       </c>
       <c r="W155" t="n">
-        <v>0.451</v>
+        <v>0.45</v>
       </c>
       <c r="X155" t="n">
-        <v>0.04</v>
+        <v>0.113</v>
       </c>
       <c r="Y155" t="n">
-        <v>0.029</v>
+        <v>0.092</v>
       </c>
       <c r="Z155" t="n">
-        <v>6.664</v>
+        <v>6.884</v>
       </c>
       <c r="AA155" t="n">
-        <v>8.869999999999999</v>
+        <v>9.082000000000001</v>
       </c>
       <c r="AB155" t="n">
-        <v>0.136</v>
+        <v>0.091</v>
       </c>
       <c r="AC155" t="n">
-        <v>0.5629999999999999</v>
+        <v>0.597</v>
       </c>
       <c r="AD155" t="n">
-        <v>0.029</v>
+        <v>0.089</v>
       </c>
     </row>
     <row r="156">
@@ -17211,16 +17211,16 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>669394</v>
+        <v>669743</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Jake Burger</t>
+          <t>Alex Call</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>Burger</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -17230,78 +17230,78 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
+          <t>LAD</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
           <t>TEX</t>
         </is>
       </c>
-      <c r="J156" t="inlineStr">
-        <is>
-          <t>LAD</t>
-        </is>
-      </c>
       <c r="K156" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L156" t="n">
-        <v>4.479</v>
+        <v>3.551</v>
       </c>
       <c r="M156" t="n">
-        <v>4.126</v>
+        <v>3.064</v>
       </c>
       <c r="N156" t="n">
-        <v>0.913</v>
+        <v>0.632</v>
       </c>
       <c r="O156" t="n">
-        <v>1.576</v>
+        <v>0.975</v>
       </c>
       <c r="P156" t="n">
-        <v>1.168</v>
+        <v>0.741</v>
       </c>
       <c r="Q156" t="n">
-        <v>0.248</v>
+        <v>0.405</v>
       </c>
       <c r="R156" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.437</v>
       </c>
       <c r="S156" t="n">
-        <v>0.192</v>
+        <v>0.117</v>
       </c>
       <c r="T156" t="n">
-        <v>0.011</v>
+        <v>0.006</v>
       </c>
       <c r="U156" t="n">
-        <v>0.15</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="V156" t="n">
-        <v>0.586</v>
+        <v>0.274</v>
       </c>
       <c r="W156" t="n">
-        <v>0.458</v>
+        <v>0.302</v>
       </c>
       <c r="X156" t="n">
-        <v>0.037</v>
+        <v>0.09</v>
       </c>
       <c r="Y156" t="n">
-        <v>0.03</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z156" t="n">
-        <v>6.96</v>
+        <v>4.971</v>
       </c>
       <c r="AA156" t="n">
-        <v>9.17</v>
+        <v>6.484</v>
       </c>
       <c r="AB156" t="n">
-        <v>0.138</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="AC156" t="n">
-        <v>0.619</v>
+        <v>0.483</v>
       </c>
       <c r="AD156" t="n">
-        <v>0.03</v>
+        <v>0.06900000000000001</v>
       </c>
     </row>
     <row r="157">
@@ -17319,21 +17319,21 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>669701</v>
+        <v>673962</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Josh Smith</t>
+          <t>Josh Jung</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>Smith</t>
+          <t>Jung</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -17355,61 +17355,61 @@
         <v>8</v>
       </c>
       <c r="L157" t="n">
-        <v>4.086</v>
+        <v>4.03</v>
       </c>
       <c r="M157" t="n">
-        <v>3.463</v>
+        <v>3.635</v>
       </c>
       <c r="N157" t="n">
-        <v>0.803</v>
+        <v>0.856</v>
       </c>
       <c r="O157" t="n">
-        <v>1.269</v>
+        <v>1.351</v>
       </c>
       <c r="P157" t="n">
-        <v>0.694</v>
+        <v>0.946</v>
       </c>
       <c r="Q157" t="n">
-        <v>0.522</v>
+        <v>0.307</v>
       </c>
       <c r="R157" t="n">
-        <v>0.522</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="S157" t="n">
-        <v>0.183</v>
+        <v>0.191</v>
       </c>
       <c r="T157" t="n">
-        <v>0.011</v>
+        <v>0.015</v>
       </c>
       <c r="U157" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.091</v>
       </c>
       <c r="V157" t="n">
-        <v>0.442</v>
+        <v>0.446</v>
       </c>
       <c r="W157" t="n">
-        <v>0.472</v>
+        <v>0.42</v>
       </c>
       <c r="X157" t="n">
-        <v>0.102</v>
+        <v>0.043</v>
       </c>
       <c r="Y157" t="n">
-        <v>0.082</v>
+        <v>0.033</v>
       </c>
       <c r="Z157" t="n">
-        <v>6.717</v>
+        <v>6.173</v>
       </c>
       <c r="AA157" t="n">
-        <v>8.917</v>
+        <v>8.074</v>
       </c>
       <c r="AB157" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="AC157" t="n">
-        <v>0.571</v>
+        <v>0.604</v>
       </c>
       <c r="AD157" t="n">
-        <v>0.079</v>
+        <v>0.033</v>
       </c>
     </row>
     <row r="158">
@@ -17427,16 +17427,16 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>673962</v>
+        <v>677649</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Josh Jung</t>
+          <t>Ezequiel Duran</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Jung</t>
+          <t>Duran</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -17463,61 +17463,61 @@
         <v>9</v>
       </c>
       <c r="L158" t="n">
-        <v>3.957</v>
+        <v>3.843</v>
       </c>
       <c r="M158" t="n">
-        <v>3.565</v>
+        <v>3.465</v>
       </c>
       <c r="N158" t="n">
-        <v>0.829</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="O158" t="n">
-        <v>1.297</v>
+        <v>1.265</v>
       </c>
       <c r="P158" t="n">
-        <v>0.886</v>
+        <v>0.867</v>
       </c>
       <c r="Q158" t="n">
-        <v>0.3</v>
+        <v>0.296</v>
       </c>
       <c r="R158" t="n">
-        <v>0.544</v>
+        <v>0.545</v>
       </c>
       <c r="S158" t="n">
-        <v>0.187</v>
+        <v>0.17</v>
       </c>
       <c r="T158" t="n">
-        <v>0.011</v>
+        <v>0.005</v>
       </c>
       <c r="U158" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.091</v>
       </c>
       <c r="V158" t="n">
-        <v>0.452</v>
+        <v>0.405</v>
       </c>
       <c r="W158" t="n">
-        <v>0.434</v>
+        <v>0.403</v>
       </c>
       <c r="X158" t="n">
-        <v>0.044</v>
+        <v>0.096</v>
       </c>
       <c r="Y158" t="n">
-        <v>0.037</v>
+        <v>0.077</v>
       </c>
       <c r="Z158" t="n">
-        <v>6.075</v>
+        <v>6.031</v>
       </c>
       <c r="AA158" t="n">
-        <v>7.981</v>
+        <v>7.852</v>
       </c>
       <c r="AB158" t="n">
-        <v>0.083</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="AC158" t="n">
-        <v>0.588</v>
+        <v>0.575</v>
       </c>
       <c r="AD158" t="n">
-        <v>0.036</v>
+        <v>0.074</v>
       </c>
     </row>
     <row r="159">
@@ -17568,64 +17568,64 @@
         </is>
       </c>
       <c r="K159" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L159" t="n">
-        <v>3.796</v>
+        <v>4.169</v>
       </c>
       <c r="M159" t="n">
-        <v>3.463</v>
+        <v>3.819</v>
       </c>
       <c r="N159" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.733</v>
       </c>
       <c r="O159" t="n">
-        <v>1.156</v>
+        <v>1.271</v>
       </c>
       <c r="P159" t="n">
-        <v>1.001</v>
+        <v>1.12</v>
       </c>
       <c r="Q159" t="n">
-        <v>0.249</v>
+        <v>0.271</v>
       </c>
       <c r="R159" t="n">
-        <v>0.433</v>
+        <v>0.443</v>
       </c>
       <c r="S159" t="n">
-        <v>0.151</v>
+        <v>0.162</v>
       </c>
       <c r="T159" t="n">
-        <v>0.003</v>
+        <v>0.008</v>
       </c>
       <c r="U159" t="n">
-        <v>0.103</v>
+        <v>0.12</v>
       </c>
       <c r="V159" t="n">
-        <v>0.363</v>
+        <v>0.399</v>
       </c>
       <c r="W159" t="n">
-        <v>0.306</v>
+        <v>0.349</v>
       </c>
       <c r="X159" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.098</v>
       </c>
       <c r="Y159" t="n">
-        <v>0.055</v>
+        <v>0.081</v>
       </c>
       <c r="Z159" t="n">
-        <v>5.215</v>
+        <v>5.846</v>
       </c>
       <c r="AA159" t="n">
-        <v>6.79</v>
+        <v>7.625</v>
       </c>
       <c r="AB159" t="n">
-        <v>0.098</v>
+        <v>0.113</v>
       </c>
       <c r="AC159" t="n">
-        <v>0.52</v>
+        <v>0.54</v>
       </c>
       <c r="AD159" t="n">
-        <v>0.054</v>
+        <v>0.077</v>
       </c>
     </row>
     <row r="160">
@@ -17643,21 +17643,21 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>690976</v>
+        <v>687221</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Alex Freeland</t>
+          <t>Dalton Rushing</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>Freeland</t>
+          <t>Rushing</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
@@ -17676,64 +17676,64 @@
         </is>
       </c>
       <c r="K160" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L160" t="n">
-        <v>3.444</v>
+        <v>3.688</v>
       </c>
       <c r="M160" t="n">
-        <v>3.074</v>
+        <v>3.376</v>
       </c>
       <c r="N160" t="n">
-        <v>0.511</v>
+        <v>0.572</v>
       </c>
       <c r="O160" t="n">
-        <v>0.828</v>
+        <v>1.034</v>
       </c>
       <c r="P160" t="n">
-        <v>1.282</v>
+        <v>1.262</v>
       </c>
       <c r="Q160" t="n">
-        <v>0.303</v>
+        <v>0.235</v>
       </c>
       <c r="R160" t="n">
-        <v>0.334</v>
+        <v>0.341</v>
       </c>
       <c r="S160" t="n">
-        <v>0.102</v>
+        <v>0.116</v>
       </c>
       <c r="T160" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="U160" t="n">
-        <v>0.065</v>
+        <v>0.115</v>
       </c>
       <c r="V160" t="n">
-        <v>0.24</v>
+        <v>0.33</v>
       </c>
       <c r="W160" t="n">
-        <v>0.306</v>
+        <v>0.296</v>
       </c>
       <c r="X160" t="n">
-        <v>0.033</v>
+        <v>0.019</v>
       </c>
       <c r="Y160" t="n">
-        <v>0.026</v>
+        <v>0.013</v>
       </c>
       <c r="Z160" t="n">
-        <v>4.068</v>
+        <v>4.542</v>
       </c>
       <c r="AA160" t="n">
-        <v>5.365</v>
+        <v>5.986</v>
       </c>
       <c r="AB160" t="n">
-        <v>0.064</v>
+        <v>0.112</v>
       </c>
       <c r="AC160" t="n">
-        <v>0.412</v>
+        <v>0.463</v>
       </c>
       <c r="AD160" t="n">
-        <v>0.025</v>
+        <v>0.013</v>
       </c>
     </row>
     <row r="161">
@@ -17751,97 +17751,97 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>694497</v>
+        <v>690976</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Evan Carter</t>
+          <t>Alex Freeland</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>Carter</t>
+          <t>Freeland</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
+          <t>LAD</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
           <t>TEX</t>
-        </is>
-      </c>
-      <c r="J161" t="inlineStr">
-        <is>
-          <t>LAD</t>
         </is>
       </c>
       <c r="K161" t="n">
         <v>6</v>
       </c>
       <c r="L161" t="n">
-        <v>4.229</v>
+        <v>3.886</v>
       </c>
       <c r="M161" t="n">
-        <v>3.524</v>
+        <v>3.465</v>
       </c>
       <c r="N161" t="n">
-        <v>0.712</v>
+        <v>0.549</v>
       </c>
       <c r="O161" t="n">
-        <v>1.165</v>
+        <v>0.893</v>
       </c>
       <c r="P161" t="n">
-        <v>0.97</v>
+        <v>1.458</v>
       </c>
       <c r="Q161" t="n">
-        <v>0.622</v>
+        <v>0.339</v>
       </c>
       <c r="R161" t="n">
-        <v>0.45</v>
+        <v>0.364</v>
       </c>
       <c r="S161" t="n">
-        <v>0.161</v>
+        <v>0.102</v>
       </c>
       <c r="T161" t="n">
-        <v>0.011</v>
+        <v>0.006</v>
       </c>
       <c r="U161" t="n">
-        <v>0.09</v>
+        <v>0.077</v>
       </c>
       <c r="V161" t="n">
-        <v>0.386</v>
+        <v>0.277</v>
       </c>
       <c r="W161" t="n">
-        <v>0.475</v>
+        <v>0.286</v>
       </c>
       <c r="X161" t="n">
-        <v>0.249</v>
+        <v>0.034</v>
       </c>
       <c r="Y161" t="n">
-        <v>0.208</v>
+        <v>0.028</v>
       </c>
       <c r="Z161" t="n">
-        <v>7.146</v>
+        <v>4.36</v>
       </c>
       <c r="AA161" t="n">
-        <v>9.476000000000001</v>
+        <v>5.747</v>
       </c>
       <c r="AB161" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.075</v>
       </c>
       <c r="AC161" t="n">
-        <v>0.525</v>
+        <v>0.439</v>
       </c>
       <c r="AD161" t="n">
-        <v>0.19</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="162">
@@ -17859,21 +17859,21 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>694671</v>
+        <v>694497</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Wyatt Langford</t>
+          <t>Evan Carter</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>Langford</t>
+          <t>Carter</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
@@ -17895,61 +17895,61 @@
         <v>2</v>
       </c>
       <c r="L162" t="n">
-        <v>4.795</v>
+        <v>4.729</v>
       </c>
       <c r="M162" t="n">
-        <v>3.922</v>
+        <v>3.892</v>
       </c>
       <c r="N162" t="n">
-        <v>0.921</v>
+        <v>0.773</v>
       </c>
       <c r="O162" t="n">
-        <v>1.648</v>
+        <v>1.254</v>
       </c>
       <c r="P162" t="n">
-        <v>1.164</v>
+        <v>1.064</v>
       </c>
       <c r="Q162" t="n">
-        <v>0.779</v>
+        <v>0.737</v>
       </c>
       <c r="R162" t="n">
-        <v>0.5669999999999999</v>
+        <v>0.496</v>
       </c>
       <c r="S162" t="n">
-        <v>0.162</v>
+        <v>0.167</v>
       </c>
       <c r="T162" t="n">
-        <v>0.013</v>
+        <v>0.016</v>
       </c>
       <c r="U162" t="n">
-        <v>0.18</v>
+        <v>0.094</v>
       </c>
       <c r="V162" t="n">
-        <v>0.542</v>
+        <v>0.387</v>
       </c>
       <c r="W162" t="n">
-        <v>0.67</v>
+        <v>0.569</v>
       </c>
       <c r="X162" t="n">
-        <v>0.275</v>
+        <v>0.286</v>
       </c>
       <c r="Y162" t="n">
-        <v>0.224</v>
+        <v>0.232</v>
       </c>
       <c r="Z162" t="n">
-        <v>9.513</v>
+        <v>7.937</v>
       </c>
       <c r="AA162" t="n">
-        <v>12.668</v>
+        <v>10.54</v>
       </c>
       <c r="AB162" t="n">
-        <v>0.165</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="AC162" t="n">
-        <v>0.626</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="AD162" t="n">
-        <v>0.206</v>
+        <v>0.204</v>
       </c>
     </row>
     <row r="163">
@@ -18000,64 +18000,64 @@
         </is>
       </c>
       <c r="K163" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L163" t="n">
-        <v>3.472</v>
+        <v>3.324</v>
       </c>
       <c r="M163" t="n">
-        <v>3.188</v>
+        <v>3.04</v>
       </c>
       <c r="N163" t="n">
-        <v>0.514</v>
+        <v>0.49</v>
       </c>
       <c r="O163" t="n">
-        <v>0.843</v>
+        <v>0.775</v>
       </c>
       <c r="P163" t="n">
-        <v>1.262</v>
+        <v>1.19</v>
       </c>
       <c r="Q163" t="n">
-        <v>0.223</v>
+        <v>0.22</v>
       </c>
       <c r="R163" t="n">
-        <v>0.33</v>
+        <v>0.327</v>
       </c>
       <c r="S163" t="n">
-        <v>0.108</v>
+        <v>0.099</v>
       </c>
       <c r="T163" t="n">
-        <v>0.008</v>
+        <v>0.005</v>
       </c>
       <c r="U163" t="n">
-        <v>0.068</v>
+        <v>0.059</v>
       </c>
       <c r="V163" t="n">
-        <v>0.242</v>
+        <v>0.211</v>
       </c>
       <c r="W163" t="n">
-        <v>0.266</v>
+        <v>0.279</v>
       </c>
       <c r="X163" t="n">
-        <v>0.155</v>
+        <v>0.158</v>
       </c>
       <c r="Y163" t="n">
-        <v>0.128</v>
+        <v>0.133</v>
       </c>
       <c r="Z163" t="n">
-        <v>4.378</v>
+        <v>4.187</v>
       </c>
       <c r="AA163" t="n">
-        <v>5.663</v>
+        <v>5.412</v>
       </c>
       <c r="AB163" t="n">
-        <v>0.066</v>
+        <v>0.058</v>
       </c>
       <c r="AC163" t="n">
-        <v>0.412</v>
+        <v>0.401</v>
       </c>
       <c r="AD163" t="n">
-        <v>0.12</v>
+        <v>0.127</v>
       </c>
     </row>
     <row r="164">

</xml_diff>